<commit_message>
[DG22-2636] adjust auto test data based on result in DEV
</commit_message>
<xml_diff>
--- a/packages/test/cypress/fixtures/data.xlsx
+++ b/packages/test/cypress/fixtures/data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/felix/kororo/repository/safeguard-github/rules-interface/packages/test/cypress/fixtures/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F8B17345-5350-E54B-B194-A1C7CAF19E4E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1A5FF970-B368-C04C-AF36-48CD45A62C5F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="38400" windowHeight="21100" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="38400" windowHeight="21100" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="D17_C" sheetId="10" r:id="rId1"/>
@@ -545,7 +545,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -558,8 +558,6 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2181,7 +2179,7 @@
     <col min="2" max="2" width="10.33203125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="30.1640625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="45.5" style="5" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="35.33203125" style="9" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="35.33203125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="9.33203125" customWidth="1"/>
     <col min="7" max="7" width="31.6640625" bestFit="1" customWidth="1"/>
   </cols>
@@ -2245,7 +2243,7 @@
       <c r="D3" s="7" t="s">
         <v>87</v>
       </c>
-      <c r="E3" s="8">
+      <c r="E3" s="3">
         <v>22</v>
       </c>
       <c r="F3" s="3">
@@ -2268,7 +2266,7 @@
       <c r="D4" s="5" t="s">
         <v>87</v>
       </c>
-      <c r="E4" s="9">
+      <c r="E4">
         <v>33</v>
       </c>
       <c r="F4">
@@ -2291,7 +2289,7 @@
       <c r="D5" s="5" t="s">
         <v>87</v>
       </c>
-      <c r="E5" s="9">
+      <c r="E5">
         <v>15</v>
       </c>
       <c r="F5">
@@ -3065,16 +3063,16 @@
         <v>79</v>
       </c>
       <c r="H3">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="I3">
-        <v>245</v>
+        <v>146</v>
       </c>
       <c r="J3">
-        <v>22.01</v>
+        <v>26.76</v>
       </c>
       <c r="K3">
-        <v>23.37</v>
+        <v>13.97</v>
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.2">
@@ -3100,13 +3098,13 @@
         <v>80</v>
       </c>
       <c r="H4">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="I4">
         <v>89</v>
       </c>
       <c r="J4">
-        <v>0</v>
+        <v>38.229999999999997</v>
       </c>
       <c r="K4">
         <v>8.65</v>
@@ -3456,30 +3454,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="ca5ba3f9-dfeb-4931-84ba-86796a0d6823">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <_ip_UnifiedCompliancePolicyUIAction xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
-    <DAte xmlns="ca5ba3f9-dfeb-4931-84ba-86796a0d6823" xsi:nil="true"/>
-    <_ip_UnifiedCompliancePolicyProperties xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
-    <date0 xmlns="ca5ba3f9-dfeb-4931-84ba-86796a0d6823" xsi:nil="true"/>
-    <TaxCatchAll xmlns="9ea08096-1d6a-4225-8886-dcb3dd04c4bd" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010001F1E234AE2DD64CAC7C4C2A8D43AD9F" ma:contentTypeVersion="23" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="6fdfd0681d808c54b86c2d268d3bba2e">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns1="http://schemas.microsoft.com/sharepoint/v3" xmlns:ns2="ca5ba3f9-dfeb-4931-84ba-86796a0d6823" xmlns:ns3="0a6f95da-2a98-4fc3-a63b-269af51b7506" xmlns:ns4="9ea08096-1d6a-4225-8886-dcb3dd04c4bd" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="5f084bf1f5a61c27721f169ac85480e0" ns1:_="" ns2:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="http://schemas.microsoft.com/sharepoint/v3"/>
@@ -3768,27 +3742,31 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3F5E14B5-D6EF-401C-82ED-6CA5F26974B2}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="ca5ba3f9-dfeb-4931-84ba-86796a0d6823"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
-    <ds:schemaRef ds:uri="9ea08096-1d6a-4225-8886-dcb3dd04c4bd"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6A69F337-BFDC-4B9A-9645-ACD2998E51C5}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="ca5ba3f9-dfeb-4931-84ba-86796a0d6823">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <_ip_UnifiedCompliancePolicyUIAction xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
+    <DAte xmlns="ca5ba3f9-dfeb-4931-84ba-86796a0d6823" xsi:nil="true"/>
+    <_ip_UnifiedCompliancePolicyProperties xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
+    <date0 xmlns="ca5ba3f9-dfeb-4931-84ba-86796a0d6823" xsi:nil="true"/>
+    <TaxCatchAll xmlns="9ea08096-1d6a-4225-8886-dcb3dd04c4bd" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4D779FCF-00EF-4E40-96D9-8E341306CAB4}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -3807,4 +3785,24 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6A69F337-BFDC-4B9A-9645-ACD2998E51C5}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3F5E14B5-D6EF-401C-82ED-6CA5F26974B2}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="ca5ba3f9-dfeb-4931-84ba-86796a0d6823"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
+    <ds:schemaRef ds:uri="9ea08096-1d6a-4225-8886-dcb3dd04c4bd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
[DG22-2636] adjust auto test data HVAC1
</commit_message>
<xml_diff>
--- a/packages/test/cypress/fixtures/data.xlsx
+++ b/packages/test/cypress/fixtures/data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/felix/kororo/repository/safeguard-github/rules-interface/packages/test/cypress/fixtures/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1A5FF970-B368-C04C-AF36-48CD45A62C5F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{915F736E-F939-424F-8CF3-70F585F785AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="38400" windowHeight="21100" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -3098,13 +3098,13 @@
         <v>80</v>
       </c>
       <c r="H4">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="I4">
         <v>89</v>
       </c>
       <c r="J4">
-        <v>38.229999999999997</v>
+        <v>0</v>
       </c>
       <c r="K4">
         <v>8.65</v>
@@ -3454,6 +3454,30 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="ca5ba3f9-dfeb-4931-84ba-86796a0d6823">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <_ip_UnifiedCompliancePolicyUIAction xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
+    <DAte xmlns="ca5ba3f9-dfeb-4931-84ba-86796a0d6823" xsi:nil="true"/>
+    <_ip_UnifiedCompliancePolicyProperties xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
+    <date0 xmlns="ca5ba3f9-dfeb-4931-84ba-86796a0d6823" xsi:nil="true"/>
+    <TaxCatchAll xmlns="9ea08096-1d6a-4225-8886-dcb3dd04c4bd" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010001F1E234AE2DD64CAC7C4C2A8D43AD9F" ma:contentTypeVersion="23" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="6fdfd0681d808c54b86c2d268d3bba2e">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns1="http://schemas.microsoft.com/sharepoint/v3" xmlns:ns2="ca5ba3f9-dfeb-4931-84ba-86796a0d6823" xmlns:ns3="0a6f95da-2a98-4fc3-a63b-269af51b7506" xmlns:ns4="9ea08096-1d6a-4225-8886-dcb3dd04c4bd" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="5f084bf1f5a61c27721f169ac85480e0" ns1:_="" ns2:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="http://schemas.microsoft.com/sharepoint/v3"/>
@@ -3742,31 +3766,27 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3F5E14B5-D6EF-401C-82ED-6CA5F26974B2}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="ca5ba3f9-dfeb-4931-84ba-86796a0d6823"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
+    <ds:schemaRef ds:uri="9ea08096-1d6a-4225-8886-dcb3dd04c4bd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="ca5ba3f9-dfeb-4931-84ba-86796a0d6823">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <_ip_UnifiedCompliancePolicyUIAction xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
-    <DAte xmlns="ca5ba3f9-dfeb-4931-84ba-86796a0d6823" xsi:nil="true"/>
-    <_ip_UnifiedCompliancePolicyProperties xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
-    <date0 xmlns="ca5ba3f9-dfeb-4931-84ba-86796a0d6823" xsi:nil="true"/>
-    <TaxCatchAll xmlns="9ea08096-1d6a-4225-8886-dcb3dd04c4bd" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6A69F337-BFDC-4B9A-9645-ACD2998E51C5}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4D779FCF-00EF-4E40-96D9-8E341306CAB4}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -3785,24 +3805,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6A69F337-BFDC-4B9A-9645-ACD2998E51C5}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3F5E14B5-D6EF-401C-82ED-6CA5F26974B2}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="ca5ba3f9-dfeb-4931-84ba-86796a0d6823"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
-    <ds:schemaRef ds:uri="9ea08096-1d6a-4225-8886-dcb3dd04c4bd"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
[DG22-2637] automate testing for pool pump and spare refrigerator eligibility
</commit_message>
<xml_diff>
--- a/packages/test/cypress/fixtures/data.xlsx
+++ b/packages/test/cypress/fixtures/data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/felix/kororo/repository/safeguard-github/rules-interface/packages/test/cypress/fixtures/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{915F736E-F939-424F-8CF3-70F585F785AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{877A4C56-E36B-E646-8B62-313F7CC6DC34}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="38400" windowHeight="21100" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="38400" windowHeight="21100" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="D17_C" sheetId="10" r:id="rId1"/>
@@ -21,11 +21,13 @@
     <sheet name="D19_C" sheetId="11" r:id="rId6"/>
     <sheet name="SYS2_D5_C" sheetId="9" r:id="rId7"/>
     <sheet name="HVAC1_C" sheetId="1" r:id="rId8"/>
-    <sheet name="HVAC1_E" sheetId="4" r:id="rId9"/>
-    <sheet name="bca-climate-zone" sheetId="2" r:id="rId10"/>
-    <sheet name="postcode" sheetId="3" r:id="rId11"/>
-    <sheet name="HVAC1_C (2)" sheetId="7" r:id="rId12"/>
-    <sheet name="HVAC1_E (2)" sheetId="8" r:id="rId13"/>
+    <sheet name="C1_E" sheetId="17" r:id="rId9"/>
+    <sheet name="SYS2_D5_E" sheetId="16" r:id="rId10"/>
+    <sheet name="HVAC1_E" sheetId="4" r:id="rId11"/>
+    <sheet name="bca-climate-zone" sheetId="2" r:id="rId12"/>
+    <sheet name="postcode" sheetId="3" r:id="rId13"/>
+    <sheet name="HVAC1_C (2)" sheetId="7" r:id="rId14"/>
+    <sheet name="HVAC1_E (2)" sheetId="8" r:id="rId15"/>
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
@@ -48,7 +50,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="526" uniqueCount="150">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="608" uniqueCount="181">
   <si>
     <t>Test ID</t>
   </si>
@@ -498,6 +500,99 @@
   </si>
   <si>
     <t>BESS2_C_001</t>
+  </si>
+  <si>
+    <t>SYS2_PDRSAug24_new_installation_or_replacement</t>
+  </si>
+  <si>
+    <t>SYS2_PDRSAug24_equipment_installed_on_site</t>
+  </si>
+  <si>
+    <t>Has the new or replacement pool pump been installed on Site?</t>
+  </si>
+  <si>
+    <t>SYS2_PDRSAug24_qualified_install_removal</t>
+  </si>
+  <si>
+    <t>SYS2_PDRSAug24_engaged_ACP</t>
+  </si>
+  <si>
+    <t>SYS2_PDRSAug24_minimum_payment</t>
+  </si>
+  <si>
+    <t>SYS2_PDRSAug24_equipment_registered_in_GEMS</t>
+  </si>
+  <si>
+    <t>Is the installed End-User equipment a registered product on the GEMS registry under GEMS (Swimming Pool Pump-units) Determination 2021?</t>
+  </si>
+  <si>
+    <t>SYS2_PDRSAug24_star_rating_minimum_four</t>
+  </si>
+  <si>
+    <t>Does the new End-User equipment have a minimum star rating of 4?</t>
+  </si>
+  <si>
+    <t>Does the new End-User equipment have a warranty of at least 3 years?</t>
+  </si>
+  <si>
+    <t>SYS2_PDRSAug24_warranty</t>
+  </si>
+  <si>
+    <t>SYS2_E_001</t>
+  </si>
+  <si>
+    <t>SYS2_E_002</t>
+  </si>
+  <si>
+    <t>SYS2_PDRSAug24_equipment_installed_on_site,SYS2_PDRSAug24_qualified_install_removal</t>
+  </si>
+  <si>
+    <t>C1_E_001</t>
+  </si>
+  <si>
+    <t>C1_E_002</t>
+  </si>
+  <si>
+    <t>Is the activity the removal of a spare non-primary refrigerator or freezer at the site?</t>
+  </si>
+  <si>
+    <t>C1_PDRSAug24_removal</t>
+  </si>
+  <si>
+    <t>Is there another refrigerator or freezer on site that provides primary refrigeration or freezing services, located in, or closer to, the kitchen?</t>
+  </si>
+  <si>
+    <t>C1_PDRSAug24_primary_refrigeration</t>
+  </si>
+  <si>
+    <t>C1_PDRSAug24_engaged_ACP</t>
+  </si>
+  <si>
+    <t>Is the End-User equipment located in a residential building?</t>
+  </si>
+  <si>
+    <t>C1_PDRSAug24_residential_building</t>
+  </si>
+  <si>
+    <t>Is the End-User equipment in working order?</t>
+  </si>
+  <si>
+    <t>C1_PDRSAug24_in_working_order</t>
+  </si>
+  <si>
+    <t>Is the End-User equipment classified as Group 1, 2, 3, 4, 5T, 5B, 5S, 6C, 6U or 7 according to AS/NZS 4474.1 and 4474.2 Performance of household electrical appliances—Refrigerating appliances?</t>
+  </si>
+  <si>
+    <t>C1_PDRSAug24_classified_group</t>
+  </si>
+  <si>
+    <t>helperC1_PDRSAug24_capacity_200_litres_or_more</t>
+  </si>
+  <si>
+    <t>C1_PDRSAug24_capacity_200_litres_or_more</t>
+  </si>
+  <si>
+    <t>C1_PDRSAug24_primary_refrigeration,C1_PDRSAug24_engaged_ACP</t>
   </si>
 </sst>
 </file>
@@ -1026,6 +1121,468 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BDE3D036-FEBF-5D43-AC42-09E358779E0F}">
+  <dimension ref="A1:K4"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="14.6640625" customWidth="1"/>
+    <col min="3" max="3" width="46.33203125" style="4" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="48.6640625" style="4" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="56.1640625" style="4" customWidth="1"/>
+    <col min="6" max="6" width="45.6640625" style="5" customWidth="1"/>
+    <col min="7" max="7" width="41" style="5" customWidth="1"/>
+    <col min="8" max="8" width="51.83203125" style="5" customWidth="1"/>
+    <col min="9" max="9" width="44.5" style="5" customWidth="1"/>
+    <col min="10" max="10" width="39.6640625" style="5" customWidth="1"/>
+    <col min="11" max="11" width="48.1640625" style="4" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:11" ht="48" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1" s="4" t="s">
+        <v>152</v>
+      </c>
+      <c r="E1" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="F1" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="G1" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1" s="4" t="s">
+        <v>157</v>
+      </c>
+      <c r="I1" s="4" t="s">
+        <v>159</v>
+      </c>
+      <c r="J1" s="4" t="s">
+        <v>160</v>
+      </c>
+      <c r="K1" s="4" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" ht="16" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B2" t="s">
+        <v>68</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>150</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>151</v>
+      </c>
+      <c r="E2" s="4" t="s">
+        <v>153</v>
+      </c>
+      <c r="F2" s="4" t="s">
+        <v>154</v>
+      </c>
+      <c r="G2" s="4" t="s">
+        <v>155</v>
+      </c>
+      <c r="H2" s="4" t="s">
+        <v>156</v>
+      </c>
+      <c r="I2" s="4" t="s">
+        <v>158</v>
+      </c>
+      <c r="J2" s="4" t="s">
+        <v>161</v>
+      </c>
+      <c r="K2" s="4" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" ht="16" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>162</v>
+      </c>
+      <c r="B3" t="s">
+        <v>69</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="F3" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="G3" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="H3" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="I3" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="J3" s="4" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" ht="32" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>163</v>
+      </c>
+      <c r="B4" t="s">
+        <v>69</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="F4" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="G4" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="H4" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="I4" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="J4" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="K4" s="4" t="s">
+        <v>164</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BE7981E0-7582-47E2-8222-6AD74E67DB3E}">
+  <sheetPr>
+    <tabColor rgb="FFFFFFFF"/>
+  </sheetPr>
+  <dimension ref="A1:P6"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="13.83203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="18" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="62.33203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="58.6640625" style="4" customWidth="1"/>
+    <col min="5" max="5" width="45.83203125" style="5" customWidth="1"/>
+    <col min="6" max="6" width="45.5" style="4" customWidth="1"/>
+    <col min="7" max="7" width="47.5" style="4" customWidth="1"/>
+    <col min="8" max="8" width="36.5" style="4" customWidth="1"/>
+    <col min="9" max="9" width="48.1640625" style="4" customWidth="1"/>
+    <col min="10" max="10" width="44.33203125" style="4" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="43.5" style="4" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="38.33203125" style="4" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="47.6640625" style="4" bestFit="1" customWidth="1"/>
+    <col min="14" max="15" width="36.5" style="4" customWidth="1"/>
+    <col min="16" max="16" width="54" style="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:16" ht="80" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="E1" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="F1" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="G1" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="H1" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="J1" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="K1" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="L1" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="M1" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="N1" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="O1" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="P1" s="1" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="2" spans="1:16" ht="16" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B2" t="s">
+        <v>68</v>
+      </c>
+      <c r="C2" t="s">
+        <v>66</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="E2" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="F2" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="G2" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="H2" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="I2" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="J2" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="K2" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="L2" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="M2" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="N2" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="O2" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="P2" s="1" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="3" spans="1:16" ht="16" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>47</v>
+      </c>
+      <c r="B3" t="s">
+        <v>69</v>
+      </c>
+      <c r="C3" t="s">
+        <v>77</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="E3" s="6" t="s">
+        <v>87</v>
+      </c>
+      <c r="F3" s="6" t="s">
+        <v>87</v>
+      </c>
+      <c r="G3" s="6" t="s">
+        <v>87</v>
+      </c>
+      <c r="H3" s="6" t="s">
+        <v>87</v>
+      </c>
+      <c r="I3" s="6" t="s">
+        <v>87</v>
+      </c>
+      <c r="J3" s="6" t="s">
+        <v>87</v>
+      </c>
+      <c r="K3" s="6"/>
+      <c r="L3" s="6" t="s">
+        <v>85</v>
+      </c>
+      <c r="M3" s="6" t="s">
+        <v>87</v>
+      </c>
+      <c r="N3" s="6" t="s">
+        <v>87</v>
+      </c>
+      <c r="O3" s="6"/>
+    </row>
+    <row r="4" spans="1:16" ht="48" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>48</v>
+      </c>
+      <c r="B4" t="s">
+        <v>69</v>
+      </c>
+      <c r="C4" t="s">
+        <v>77</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="E4" s="6" t="s">
+        <v>87</v>
+      </c>
+      <c r="F4" s="6" t="s">
+        <v>87</v>
+      </c>
+      <c r="G4" s="6" t="s">
+        <v>87</v>
+      </c>
+      <c r="H4" s="6" t="s">
+        <v>87</v>
+      </c>
+      <c r="I4" s="6" t="s">
+        <v>86</v>
+      </c>
+      <c r="J4" s="6"/>
+      <c r="K4" s="6" t="s">
+        <v>86</v>
+      </c>
+      <c r="L4" s="6" t="s">
+        <v>85</v>
+      </c>
+      <c r="M4" s="6" t="s">
+        <v>86</v>
+      </c>
+      <c r="N4" s="6"/>
+      <c r="O4" s="6" t="s">
+        <v>87</v>
+      </c>
+      <c r="P4" s="1" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="5" spans="1:16" ht="16" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>49</v>
+      </c>
+      <c r="B5" t="s">
+        <v>69</v>
+      </c>
+      <c r="C5" t="s">
+        <v>77</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="E5" s="6" t="s">
+        <v>87</v>
+      </c>
+      <c r="F5" s="6" t="s">
+        <v>87</v>
+      </c>
+      <c r="G5" s="6" t="s">
+        <v>87</v>
+      </c>
+      <c r="H5" s="6" t="s">
+        <v>87</v>
+      </c>
+      <c r="I5" s="6" t="s">
+        <v>87</v>
+      </c>
+      <c r="J5" s="6" t="s">
+        <v>87</v>
+      </c>
+      <c r="K5" s="6"/>
+      <c r="L5" s="6" t="s">
+        <v>85</v>
+      </c>
+      <c r="M5" s="6" t="s">
+        <v>87</v>
+      </c>
+      <c r="N5" s="6"/>
+      <c r="O5" s="6"/>
+    </row>
+    <row r="6" spans="1:16" ht="16" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
+        <v>50</v>
+      </c>
+      <c r="B6" t="s">
+        <v>69</v>
+      </c>
+      <c r="C6" t="s">
+        <v>77</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="E6" s="6" t="s">
+        <v>87</v>
+      </c>
+      <c r="F6" s="6" t="s">
+        <v>87</v>
+      </c>
+      <c r="G6" s="6" t="s">
+        <v>87</v>
+      </c>
+      <c r="H6" s="6" t="s">
+        <v>87</v>
+      </c>
+      <c r="I6" s="6" t="s">
+        <v>87</v>
+      </c>
+      <c r="J6" s="6" t="s">
+        <v>87</v>
+      </c>
+      <c r="K6" s="6"/>
+      <c r="L6" s="6" t="s">
+        <v>85</v>
+      </c>
+      <c r="M6" s="6" t="s">
+        <v>87</v>
+      </c>
+      <c r="N6" s="6" t="s">
+        <v>87</v>
+      </c>
+      <c r="O6" s="6"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2786CED2-7BEF-4054-842D-DA68BCCB8D75}">
   <dimension ref="A1:B19"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
@@ -1191,7 +1748,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B6EC151F-5CD6-4BE1-BB25-71A93C50E291}">
   <dimension ref="A1:B24"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
@@ -1397,7 +1954,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3B9C1EEA-4954-8E44-9208-CE3F5C52B99D}">
   <dimension ref="A1:K9"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
@@ -1731,7 +2288,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{60EBEADA-E54E-3C4F-9EFA-55641646C71D}">
   <sheetPr>
     <tabColor rgb="FFFFFFFF"/>
@@ -3151,302 +3708,145 @@
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BE7981E0-7582-47E2-8222-6AD74E67DB3E}">
-  <sheetPr>
-    <tabColor rgb="FFFFFFFF"/>
-  </sheetPr>
-  <dimension ref="A1:P6"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2B45B736-35F4-404E-994E-F08E1074E335}">
+  <dimension ref="A1:J4"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="13.83203125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="18" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="62.33203125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="58.6640625" style="4" customWidth="1"/>
-    <col min="5" max="5" width="45.83203125" style="5" customWidth="1"/>
-    <col min="6" max="6" width="45.5" style="4" customWidth="1"/>
-    <col min="7" max="7" width="47.5" style="4" customWidth="1"/>
-    <col min="8" max="8" width="36.5" style="4" customWidth="1"/>
-    <col min="9" max="9" width="48.1640625" style="4" customWidth="1"/>
-    <col min="10" max="10" width="44.33203125" style="4" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="43.5" style="4" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="38.33203125" style="4" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="47.6640625" style="4" bestFit="1" customWidth="1"/>
-    <col min="14" max="15" width="36.5" style="4" customWidth="1"/>
-    <col min="16" max="16" width="54" style="1" customWidth="1"/>
+    <col min="1" max="1" width="14.6640625" customWidth="1"/>
+    <col min="3" max="3" width="46.33203125" style="4" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="48.6640625" style="4" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="56.1640625" style="4" customWidth="1"/>
+    <col min="6" max="6" width="45.6640625" style="5" customWidth="1"/>
+    <col min="7" max="7" width="41" style="5" customWidth="1"/>
+    <col min="8" max="8" width="51.83203125" style="5" customWidth="1"/>
+    <col min="9" max="9" width="44.5" style="5" customWidth="1"/>
+    <col min="10" max="10" width="48.1640625" style="4" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" ht="80" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:10" ht="48" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
-        <v>22</v>
+      <c r="C1" s="4" t="s">
+        <v>167</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="E1" s="5" t="s">
-        <v>24</v>
+        <v>169</v>
+      </c>
+      <c r="E1" s="4" t="s">
+        <v>25</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>25</v>
+        <v>172</v>
       </c>
       <c r="G1" s="4" t="s">
-        <v>26</v>
+        <v>174</v>
       </c>
       <c r="H1" s="4" t="s">
-        <v>27</v>
+        <v>176</v>
       </c>
       <c r="I1" s="4" t="s">
-        <v>28</v>
+        <v>178</v>
       </c>
       <c r="J1" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="K1" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="L1" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="M1" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="N1" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="O1" s="4" t="s">
-        <v>34</v>
-      </c>
-      <c r="P1" s="1" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="2" spans="1:16" ht="16" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>12</v>
       </c>
       <c r="B2" t="s">
         <v>68</v>
       </c>
-      <c r="C2" t="s">
-        <v>66</v>
+      <c r="C2" s="4" t="s">
+        <v>168</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>36</v>
-      </c>
-      <c r="E2" s="5" t="s">
-        <v>37</v>
+        <v>170</v>
+      </c>
+      <c r="E2" s="4" t="s">
+        <v>171</v>
       </c>
       <c r="F2" s="4" t="s">
-        <v>38</v>
+        <v>173</v>
       </c>
       <c r="G2" s="4" t="s">
-        <v>39</v>
+        <v>175</v>
       </c>
       <c r="H2" s="4" t="s">
-        <v>40</v>
+        <v>177</v>
       </c>
       <c r="I2" s="4" t="s">
-        <v>41</v>
+        <v>179</v>
       </c>
       <c r="J2" s="4" t="s">
-        <v>42</v>
-      </c>
-      <c r="K2" s="4" t="s">
-        <v>43</v>
-      </c>
-      <c r="L2" s="4" t="s">
-        <v>67</v>
-      </c>
-      <c r="M2" s="4" t="s">
-        <v>44</v>
-      </c>
-      <c r="N2" s="4" t="s">
-        <v>45</v>
-      </c>
-      <c r="O2" s="4" t="s">
-        <v>46</v>
-      </c>
-      <c r="P2" s="1" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="3" spans="1:16" ht="16" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>47</v>
+        <v>165</v>
       </c>
       <c r="B3" t="s">
         <v>69</v>
       </c>
-      <c r="C3" t="s">
-        <v>77</v>
+      <c r="C3" s="4" t="s">
+        <v>87</v>
       </c>
       <c r="D3" s="4" t="s">
         <v>87</v>
       </c>
-      <c r="E3" s="6" t="s">
-        <v>87</v>
-      </c>
-      <c r="F3" s="6" t="s">
-        <v>87</v>
-      </c>
-      <c r="G3" s="6" t="s">
-        <v>87</v>
-      </c>
-      <c r="H3" s="6" t="s">
-        <v>87</v>
-      </c>
-      <c r="I3" s="6" t="s">
-        <v>87</v>
-      </c>
-      <c r="J3" s="6" t="s">
-        <v>87</v>
-      </c>
-      <c r="K3" s="6"/>
-      <c r="L3" s="6" t="s">
-        <v>85</v>
-      </c>
-      <c r="M3" s="6" t="s">
-        <v>87</v>
-      </c>
-      <c r="N3" s="6" t="s">
-        <v>87</v>
-      </c>
-      <c r="O3" s="6"/>
-    </row>
-    <row r="4" spans="1:16" ht="48" x14ac:dyDescent="0.2">
+      <c r="E3" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="F3" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="G3" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="H3" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="I3" s="4" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" ht="32" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>48</v>
+        <v>166</v>
       </c>
       <c r="B4" t="s">
         <v>69</v>
       </c>
-      <c r="C4" t="s">
-        <v>77</v>
+      <c r="C4" s="4" t="s">
+        <v>87</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="E4" s="6" t="s">
-        <v>87</v>
-      </c>
-      <c r="F4" s="6" t="s">
-        <v>87</v>
-      </c>
-      <c r="G4" s="6" t="s">
-        <v>87</v>
-      </c>
-      <c r="H4" s="6" t="s">
-        <v>87</v>
-      </c>
-      <c r="I4" s="6" t="s">
         <v>86</v>
       </c>
-      <c r="J4" s="6"/>
-      <c r="K4" s="6" t="s">
+      <c r="E4" s="4" t="s">
         <v>86</v>
       </c>
-      <c r="L4" s="6" t="s">
-        <v>85</v>
-      </c>
-      <c r="M4" s="6" t="s">
-        <v>86</v>
-      </c>
-      <c r="N4" s="6"/>
-      <c r="O4" s="6" t="s">
-        <v>87</v>
-      </c>
-      <c r="P4" s="1" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="5" spans="1:16" ht="16" x14ac:dyDescent="0.2">
-      <c r="A5" t="s">
-        <v>49</v>
-      </c>
-      <c r="B5" t="s">
-        <v>69</v>
-      </c>
-      <c r="C5" t="s">
-        <v>77</v>
-      </c>
-      <c r="D5" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="E5" s="6" t="s">
-        <v>87</v>
-      </c>
-      <c r="F5" s="6" t="s">
-        <v>87</v>
-      </c>
-      <c r="G5" s="6" t="s">
-        <v>87</v>
-      </c>
-      <c r="H5" s="6" t="s">
-        <v>87</v>
-      </c>
-      <c r="I5" s="6" t="s">
-        <v>87</v>
-      </c>
-      <c r="J5" s="6" t="s">
-        <v>87</v>
-      </c>
-      <c r="K5" s="6"/>
-      <c r="L5" s="6" t="s">
-        <v>85</v>
-      </c>
-      <c r="M5" s="6" t="s">
-        <v>87</v>
-      </c>
-      <c r="N5" s="6"/>
-      <c r="O5" s="6"/>
-    </row>
-    <row r="6" spans="1:16" ht="16" x14ac:dyDescent="0.2">
-      <c r="A6" t="s">
-        <v>50</v>
-      </c>
-      <c r="B6" t="s">
-        <v>69</v>
-      </c>
-      <c r="C6" t="s">
-        <v>77</v>
-      </c>
-      <c r="D6" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="E6" s="6" t="s">
-        <v>87</v>
-      </c>
-      <c r="F6" s="6" t="s">
-        <v>87</v>
-      </c>
-      <c r="G6" s="6" t="s">
-        <v>87</v>
-      </c>
-      <c r="H6" s="6" t="s">
-        <v>87</v>
-      </c>
-      <c r="I6" s="6" t="s">
-        <v>87</v>
-      </c>
-      <c r="J6" s="6" t="s">
-        <v>87</v>
-      </c>
-      <c r="K6" s="6"/>
-      <c r="L6" s="6" t="s">
-        <v>85</v>
-      </c>
-      <c r="M6" s="6" t="s">
-        <v>87</v>
-      </c>
-      <c r="N6" s="6" t="s">
-        <v>87</v>
-      </c>
-      <c r="O6" s="6"/>
+      <c r="F4" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="G4" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="H4" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="I4" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="J4" s="4" t="s">
+        <v>180</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -3454,30 +3854,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="ca5ba3f9-dfeb-4931-84ba-86796a0d6823">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <_ip_UnifiedCompliancePolicyUIAction xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
-    <DAte xmlns="ca5ba3f9-dfeb-4931-84ba-86796a0d6823" xsi:nil="true"/>
-    <_ip_UnifiedCompliancePolicyProperties xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
-    <date0 xmlns="ca5ba3f9-dfeb-4931-84ba-86796a0d6823" xsi:nil="true"/>
-    <TaxCatchAll xmlns="9ea08096-1d6a-4225-8886-dcb3dd04c4bd" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010001F1E234AE2DD64CAC7C4C2A8D43AD9F" ma:contentTypeVersion="23" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="6fdfd0681d808c54b86c2d268d3bba2e">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns1="http://schemas.microsoft.com/sharepoint/v3" xmlns:ns2="ca5ba3f9-dfeb-4931-84ba-86796a0d6823" xmlns:ns3="0a6f95da-2a98-4fc3-a63b-269af51b7506" xmlns:ns4="9ea08096-1d6a-4225-8886-dcb3dd04c4bd" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="5f084bf1f5a61c27721f169ac85480e0" ns1:_="" ns2:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="http://schemas.microsoft.com/sharepoint/v3"/>
@@ -3766,27 +4142,31 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3F5E14B5-D6EF-401C-82ED-6CA5F26974B2}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="ca5ba3f9-dfeb-4931-84ba-86796a0d6823"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
-    <ds:schemaRef ds:uri="9ea08096-1d6a-4225-8886-dcb3dd04c4bd"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6A69F337-BFDC-4B9A-9645-ACD2998E51C5}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="ca5ba3f9-dfeb-4931-84ba-86796a0d6823">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <_ip_UnifiedCompliancePolicyUIAction xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
+    <DAte xmlns="ca5ba3f9-dfeb-4931-84ba-86796a0d6823" xsi:nil="true"/>
+    <_ip_UnifiedCompliancePolicyProperties xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
+    <date0 xmlns="ca5ba3f9-dfeb-4931-84ba-86796a0d6823" xsi:nil="true"/>
+    <TaxCatchAll xmlns="9ea08096-1d6a-4225-8886-dcb3dd04c4bd" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4D779FCF-00EF-4E40-96D9-8E341306CAB4}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -3805,4 +4185,24 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6A69F337-BFDC-4B9A-9645-ACD2998E51C5}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3F5E14B5-D6EF-401C-82ED-6CA5F26974B2}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="ca5ba3f9-dfeb-4931-84ba-86796a0d6823"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
+    <ds:schemaRef ds:uri="9ea08096-1d6a-4225-8886-dcb3dd04c4bd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
[DG22-2637] adjust auto testing data
</commit_message>
<xml_diff>
--- a/packages/test/cypress/fixtures/data.xlsx
+++ b/packages/test/cypress/fixtures/data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/felix/kororo/repository/safeguard-github/rules-interface/packages/test/cypress/fixtures/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C96FB188-7BD4-434C-8B5B-33C3B816BAA2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8BF5C672-E556-0641-B7F3-F46B8690FADC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="180" yWindow="500" windowWidth="21060" windowHeight="21040" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="7220" yWindow="2800" windowWidth="27560" windowHeight="21040" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="D17_C" sheetId="10" r:id="rId1"/>
@@ -5622,7 +5622,7 @@
         <v>23</v>
       </c>
       <c r="I3">
-        <v>245</v>
+        <v>146</v>
       </c>
       <c r="J3">
         <v>21.37</v>
@@ -5853,18 +5853,12 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="ca5ba3f9-dfeb-4931-84ba-86796a0d6823">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <_ip_UnifiedCompliancePolicyUIAction xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
-    <DAte xmlns="ca5ba3f9-dfeb-4931-84ba-86796a0d6823" xsi:nil="true"/>
-    <_ip_UnifiedCompliancePolicyProperties xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
-    <date0 xmlns="ca5ba3f9-dfeb-4931-84ba-86796a0d6823" xsi:nil="true"/>
-    <TaxCatchAll xmlns="9ea08096-1d6a-4225-8886-dcb3dd04c4bd" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -6157,22 +6151,24 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="ca5ba3f9-dfeb-4931-84ba-86796a0d6823">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <_ip_UnifiedCompliancePolicyUIAction xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
+    <DAte xmlns="ca5ba3f9-dfeb-4931-84ba-86796a0d6823" xsi:nil="true"/>
+    <_ip_UnifiedCompliancePolicyProperties xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
+    <date0 xmlns="ca5ba3f9-dfeb-4931-84ba-86796a0d6823" xsi:nil="true"/>
+    <TaxCatchAll xmlns="9ea08096-1d6a-4225-8886-dcb3dd04c4bd" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3F5E14B5-D6EF-401C-82ED-6CA5F26974B2}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6A69F337-BFDC-4B9A-9645-ACD2998E51C5}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="ca5ba3f9-dfeb-4931-84ba-86796a0d6823"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
-    <ds:schemaRef ds:uri="9ea08096-1d6a-4225-8886-dcb3dd04c4bd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -6199,9 +6195,13 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6A69F337-BFDC-4B9A-9645-ACD2998E51C5}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3F5E14B5-D6EF-401C-82ED-6CA5F26974B2}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="ca5ba3f9-dfeb-4931-84ba-86796a0d6823"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
+    <ds:schemaRef ds:uri="9ea08096-1d6a-4225-8886-dcb3dd04c4bd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
[DG22-2637] update data fixture and github workflow for test in dev
</commit_message>
<xml_diff>
--- a/packages/test/cypress/fixtures/data.xlsx
+++ b/packages/test/cypress/fixtures/data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/felix/kororo/repository/safeguard-github/rules-interface/packages/test/cypress/fixtures/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8BF5C672-E556-0641-B7F3-F46B8690FADC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E26A880D-A61A-BA43-87BC-74D35C80B635}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="7220" yWindow="2800" windowWidth="27560" windowHeight="21040" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="38400" windowHeight="21100" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="D17_C" sheetId="10" r:id="rId1"/>
@@ -5622,7 +5622,7 @@
         <v>23</v>
       </c>
       <c r="I3">
-        <v>146</v>
+        <v>245</v>
       </c>
       <c r="J3">
         <v>21.37</v>

</xml_diff>

<commit_message>
[DG22-2637] add step to upload artifacts for debugging purpose, especially the hvac1
</commit_message>
<xml_diff>
--- a/packages/test/cypress/fixtures/data.xlsx
+++ b/packages/test/cypress/fixtures/data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/felix/kororo/repository/safeguard-github/rules-interface/packages/test/cypress/fixtures/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E26A880D-A61A-BA43-87BC-74D35C80B635}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A9401C57-A73B-A048-823B-BADE772CBBC4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="38400" windowHeight="21100" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -5853,12 +5853,18 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="ca5ba3f9-dfeb-4931-84ba-86796a0d6823">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <_ip_UnifiedCompliancePolicyUIAction xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
+    <DAte xmlns="ca5ba3f9-dfeb-4931-84ba-86796a0d6823" xsi:nil="true"/>
+    <_ip_UnifiedCompliancePolicyProperties xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
+    <date0 xmlns="ca5ba3f9-dfeb-4931-84ba-86796a0d6823" xsi:nil="true"/>
+    <TaxCatchAll xmlns="9ea08096-1d6a-4225-8886-dcb3dd04c4bd" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -6151,24 +6157,22 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="ca5ba3f9-dfeb-4931-84ba-86796a0d6823">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <_ip_UnifiedCompliancePolicyUIAction xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
-    <DAte xmlns="ca5ba3f9-dfeb-4931-84ba-86796a0d6823" xsi:nil="true"/>
-    <_ip_UnifiedCompliancePolicyProperties xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
-    <date0 xmlns="ca5ba3f9-dfeb-4931-84ba-86796a0d6823" xsi:nil="true"/>
-    <TaxCatchAll xmlns="9ea08096-1d6a-4225-8886-dcb3dd04c4bd" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6A69F337-BFDC-4B9A-9645-ACD2998E51C5}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3F5E14B5-D6EF-401C-82ED-6CA5F26974B2}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="ca5ba3f9-dfeb-4931-84ba-86796a0d6823"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
+    <ds:schemaRef ds:uri="9ea08096-1d6a-4225-8886-dcb3dd04c4bd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -6195,13 +6199,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3F5E14B5-D6EF-401C-82ED-6CA5F26974B2}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6A69F337-BFDC-4B9A-9645-ACD2998E51C5}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="ca5ba3f9-dfeb-4931-84ba-86796a0d6823"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
-    <ds:schemaRef ds:uri="9ea08096-1d6a-4225-8886-dcb3dd04c4bd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
[DG22-2637] fixing the way to render postcode and bca climate zone field, and certificate result element too.
</commit_message>
<xml_diff>
--- a/packages/test/cypress/fixtures/data.xlsx
+++ b/packages/test/cypress/fixtures/data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/felix/kororo/repository/safeguard-github/rules-interface/packages/test/cypress/fixtures/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A9401C57-A73B-A048-823B-BADE772CBBC4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3C12D2BE-FDEE-EC4B-B60B-DB235242085A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="38400" windowHeight="21100" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,15 +21,15 @@
     <sheet name="D19_C" sheetId="11" r:id="rId6"/>
     <sheet name="SYS2_D5_C" sheetId="9" r:id="rId7"/>
     <sheet name="HVAC1_C" sheetId="1" r:id="rId8"/>
-    <sheet name="C1_E" sheetId="17" r:id="rId9"/>
-    <sheet name="BESS2_E" sheetId="18" r:id="rId10"/>
-    <sheet name="CORE_E" sheetId="19" r:id="rId11"/>
-    <sheet name="D17_E" sheetId="20" r:id="rId12"/>
-    <sheet name="D18_E" sheetId="22" r:id="rId13"/>
-    <sheet name="D19_E" sheetId="21" r:id="rId14"/>
-    <sheet name="D20_E" sheetId="23" r:id="rId15"/>
-    <sheet name="SYS2_D5_E" sheetId="16" r:id="rId16"/>
-    <sheet name="HVAC1_E" sheetId="4" r:id="rId17"/>
+    <sheet name="CORE_E" sheetId="19" r:id="rId9"/>
+    <sheet name="HVAC1_E" sheetId="4" r:id="rId10"/>
+    <sheet name="SYS2_D5_E" sheetId="16" r:id="rId11"/>
+    <sheet name="C1_E" sheetId="17" r:id="rId12"/>
+    <sheet name="D17_E" sheetId="20" r:id="rId13"/>
+    <sheet name="D18_E" sheetId="22" r:id="rId14"/>
+    <sheet name="D19_E" sheetId="21" r:id="rId15"/>
+    <sheet name="D20_E" sheetId="23" r:id="rId16"/>
+    <sheet name="BESS2_E" sheetId="18" r:id="rId17"/>
     <sheet name="bca-climate-zone" sheetId="2" r:id="rId18"/>
     <sheet name="postcode" sheetId="3" r:id="rId19"/>
     <sheet name="HVAC1_C (2)" sheetId="7" r:id="rId20"/>
@@ -1514,1771 +1514,6 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{521E381E-94A1-CA4C-9D15-5BDDF952F7C7}">
-  <dimension ref="A1:O4"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
-  <cols>
-    <col min="1" max="1" width="14.6640625" customWidth="1"/>
-    <col min="3" max="3" width="46.33203125" style="4" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="48.6640625" style="4" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="56.1640625" style="4" customWidth="1"/>
-    <col min="6" max="6" width="45.6640625" style="5" customWidth="1"/>
-    <col min="7" max="7" width="41" style="5" customWidth="1"/>
-    <col min="8" max="8" width="51.83203125" style="5" customWidth="1"/>
-    <col min="9" max="14" width="44.5" style="5" customWidth="1"/>
-    <col min="15" max="15" width="48.1640625" style="4" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:15" ht="48" x14ac:dyDescent="0.2">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="4" t="s">
-        <v>183</v>
-      </c>
-      <c r="D1" s="4" t="s">
-        <v>185</v>
-      </c>
-      <c r="E1" s="4" t="s">
-        <v>187</v>
-      </c>
-      <c r="F1" s="4" t="s">
-        <v>189</v>
-      </c>
-      <c r="G1" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="H1" s="4" t="s">
-        <v>192</v>
-      </c>
-      <c r="I1" s="4" t="s">
-        <v>194</v>
-      </c>
-      <c r="J1" s="4" t="s">
-        <v>196</v>
-      </c>
-      <c r="K1" s="4" t="s">
-        <v>198</v>
-      </c>
-      <c r="L1" s="4" t="s">
-        <v>200</v>
-      </c>
-      <c r="M1" s="4" t="s">
-        <v>202</v>
-      </c>
-      <c r="N1" s="4" t="s">
-        <v>204</v>
-      </c>
-      <c r="O1" s="4" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="2" spans="1:15" ht="32" x14ac:dyDescent="0.2">
-      <c r="A2" t="s">
-        <v>12</v>
-      </c>
-      <c r="B2" t="s">
-        <v>68</v>
-      </c>
-      <c r="C2" s="4" t="s">
-        <v>184</v>
-      </c>
-      <c r="D2" s="4" t="s">
-        <v>186</v>
-      </c>
-      <c r="E2" s="4" t="s">
-        <v>188</v>
-      </c>
-      <c r="F2" s="4" t="s">
-        <v>190</v>
-      </c>
-      <c r="G2" s="4" t="s">
-        <v>191</v>
-      </c>
-      <c r="H2" s="4" t="s">
-        <v>193</v>
-      </c>
-      <c r="I2" s="4" t="s">
-        <v>195</v>
-      </c>
-      <c r="J2" s="4" t="s">
-        <v>197</v>
-      </c>
-      <c r="K2" s="4" t="s">
-        <v>199</v>
-      </c>
-      <c r="L2" s="4" t="s">
-        <v>201</v>
-      </c>
-      <c r="M2" s="4" t="s">
-        <v>203</v>
-      </c>
-      <c r="N2" s="4" t="s">
-        <v>205</v>
-      </c>
-      <c r="O2" s="4" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="3" spans="1:15" ht="16" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
-        <v>181</v>
-      </c>
-      <c r="B3" t="s">
-        <v>69</v>
-      </c>
-      <c r="C3" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="D3" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="E3" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="F3" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="G3" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="H3" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="I3" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="J3" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="K3" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="L3" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="M3" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="N3" s="4" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="4" spans="1:15" ht="32" x14ac:dyDescent="0.2">
-      <c r="A4" t="s">
-        <v>182</v>
-      </c>
-      <c r="B4" t="s">
-        <v>69</v>
-      </c>
-      <c r="C4" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="D4" s="4" t="s">
-        <v>86</v>
-      </c>
-      <c r="E4" s="4" t="s">
-        <v>86</v>
-      </c>
-      <c r="F4" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="G4" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="H4" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="I4" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="J4" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="K4" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="L4" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="M4" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="N4" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="O4" s="4" t="s">
-        <v>206</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{97A1D2A4-B682-FE42-B308-482711D73604}">
-  <dimension ref="A1:S10"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
-  <cols>
-    <col min="1" max="1" width="14.6640625" customWidth="1"/>
-    <col min="3" max="3" width="46.33203125" style="4" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="48.6640625" style="4" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="56.1640625" style="4" customWidth="1"/>
-    <col min="6" max="6" width="45.6640625" style="5" customWidth="1"/>
-    <col min="7" max="7" width="41" style="5" customWidth="1"/>
-    <col min="8" max="8" width="51.83203125" style="5" customWidth="1"/>
-    <col min="9" max="18" width="44.5" style="5" customWidth="1"/>
-    <col min="19" max="19" width="48.1640625" style="4" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:19" ht="64" x14ac:dyDescent="0.2">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="4" t="s">
-        <v>209</v>
-      </c>
-      <c r="D1" s="4" t="s">
-        <v>211</v>
-      </c>
-      <c r="E1" s="4" t="s">
-        <v>213</v>
-      </c>
-      <c r="F1" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="G1" s="4" t="s">
-        <v>216</v>
-      </c>
-      <c r="H1" s="4" t="s">
-        <v>218</v>
-      </c>
-      <c r="I1" s="4" t="s">
-        <v>220</v>
-      </c>
-      <c r="J1" s="4" t="s">
-        <v>222</v>
-      </c>
-      <c r="K1" s="4" t="s">
-        <v>224</v>
-      </c>
-      <c r="L1" s="4" t="s">
-        <v>226</v>
-      </c>
-      <c r="M1" s="4" t="s">
-        <v>228</v>
-      </c>
-      <c r="N1" s="4" t="s">
-        <v>234</v>
-      </c>
-      <c r="O1" s="4" t="s">
-        <v>230</v>
-      </c>
-      <c r="P1" s="4" t="s">
-        <v>232</v>
-      </c>
-      <c r="Q1" s="4" t="s">
-        <v>236</v>
-      </c>
-      <c r="R1" s="4" t="s">
-        <v>238</v>
-      </c>
-      <c r="S1" s="4" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="2" spans="1:19" ht="16" x14ac:dyDescent="0.2">
-      <c r="A2" t="s">
-        <v>12</v>
-      </c>
-      <c r="B2" t="s">
-        <v>68</v>
-      </c>
-      <c r="C2" s="4" t="s">
-        <v>210</v>
-      </c>
-      <c r="D2" s="4" t="s">
-        <v>212</v>
-      </c>
-      <c r="E2" s="4" t="s">
-        <v>214</v>
-      </c>
-      <c r="F2" s="4" t="s">
-        <v>215</v>
-      </c>
-      <c r="G2" s="4" t="s">
-        <v>217</v>
-      </c>
-      <c r="H2" s="4" t="s">
-        <v>219</v>
-      </c>
-      <c r="I2" s="4" t="s">
-        <v>221</v>
-      </c>
-      <c r="J2" s="4" t="s">
-        <v>223</v>
-      </c>
-      <c r="K2" s="4" t="s">
-        <v>225</v>
-      </c>
-      <c r="L2" s="4" t="s">
-        <v>227</v>
-      </c>
-      <c r="M2" s="4" t="s">
-        <v>229</v>
-      </c>
-      <c r="N2" s="4" t="s">
-        <v>235</v>
-      </c>
-      <c r="O2" s="4" t="s">
-        <v>231</v>
-      </c>
-      <c r="P2" s="4" t="s">
-        <v>233</v>
-      </c>
-      <c r="Q2" s="4" t="s">
-        <v>237</v>
-      </c>
-      <c r="R2" s="4" t="s">
-        <v>239</v>
-      </c>
-      <c r="S2" s="4" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="3" spans="1:19" ht="16" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
-        <v>207</v>
-      </c>
-      <c r="B3" t="s">
-        <v>69</v>
-      </c>
-      <c r="C3" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="D3" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="E3" s="4" t="s">
-        <v>240</v>
-      </c>
-      <c r="F3" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="G3" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="H3" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="I3" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="J3" s="4" t="s">
-        <v>86</v>
-      </c>
-      <c r="K3" s="4" t="s">
-        <v>86</v>
-      </c>
-      <c r="L3" s="4" t="s">
-        <v>86</v>
-      </c>
-      <c r="M3" s="4" t="s">
-        <v>86</v>
-      </c>
-      <c r="N3" s="4"/>
-      <c r="O3" s="4" t="s">
-        <v>86</v>
-      </c>
-      <c r="P3" s="4" t="s">
-        <v>86</v>
-      </c>
-      <c r="Q3" s="4"/>
-      <c r="R3" s="4"/>
-    </row>
-    <row r="4" spans="1:19" ht="32" x14ac:dyDescent="0.2">
-      <c r="A4" t="s">
-        <v>208</v>
-      </c>
-      <c r="B4" t="s">
-        <v>69</v>
-      </c>
-      <c r="C4" s="4" t="s">
-        <v>86</v>
-      </c>
-      <c r="D4" s="4" t="s">
-        <v>86</v>
-      </c>
-      <c r="E4" s="4" t="s">
-        <v>240</v>
-      </c>
-      <c r="F4" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="G4" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="H4" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="I4" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="J4" s="4" t="s">
-        <v>86</v>
-      </c>
-      <c r="K4" s="4" t="s">
-        <v>86</v>
-      </c>
-      <c r="L4" s="4" t="s">
-        <v>86</v>
-      </c>
-      <c r="M4" s="4" t="s">
-        <v>86</v>
-      </c>
-      <c r="N4" s="4"/>
-      <c r="O4" s="4" t="s">
-        <v>86</v>
-      </c>
-      <c r="P4" s="4" t="s">
-        <v>86</v>
-      </c>
-      <c r="Q4" s="4"/>
-      <c r="R4" s="4"/>
-      <c r="S4" s="4" t="s">
-        <v>241</v>
-      </c>
-    </row>
-    <row r="5" spans="1:19" ht="16" x14ac:dyDescent="0.2">
-      <c r="A5" t="s">
-        <v>242</v>
-      </c>
-      <c r="B5" t="s">
-        <v>69</v>
-      </c>
-      <c r="C5" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="D5" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="E5" s="4" t="s">
-        <v>240</v>
-      </c>
-      <c r="F5" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="G5" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="H5" s="4" t="s">
-        <v>86</v>
-      </c>
-      <c r="I5" s="4"/>
-      <c r="K5" s="4" t="s">
-        <v>86</v>
-      </c>
-      <c r="L5" s="4" t="s">
-        <v>86</v>
-      </c>
-      <c r="M5" s="4" t="s">
-        <v>86</v>
-      </c>
-      <c r="O5" s="4" t="s">
-        <v>86</v>
-      </c>
-      <c r="P5" s="5" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="6" spans="1:19" ht="32" x14ac:dyDescent="0.2">
-      <c r="A6" t="s">
-        <v>243</v>
-      </c>
-      <c r="B6" t="s">
-        <v>69</v>
-      </c>
-      <c r="C6" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="D6" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="E6" s="4" t="s">
-        <v>240</v>
-      </c>
-      <c r="F6" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="G6" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="H6" s="5" t="s">
-        <v>87</v>
-      </c>
-      <c r="I6" s="5" t="s">
-        <v>86</v>
-      </c>
-      <c r="J6" s="5" t="s">
-        <v>87</v>
-      </c>
-      <c r="K6" s="5" t="s">
-        <v>86</v>
-      </c>
-      <c r="L6" s="5" t="s">
-        <v>86</v>
-      </c>
-      <c r="M6" s="5" t="s">
-        <v>86</v>
-      </c>
-      <c r="O6" s="5" t="s">
-        <v>86</v>
-      </c>
-      <c r="P6" s="5" t="s">
-        <v>86</v>
-      </c>
-      <c r="S6" s="4" t="s">
-        <v>244</v>
-      </c>
-    </row>
-    <row r="7" spans="1:19" ht="32" x14ac:dyDescent="0.2">
-      <c r="A7" t="s">
-        <v>245</v>
-      </c>
-      <c r="B7" t="s">
-        <v>69</v>
-      </c>
-      <c r="C7" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="D7" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="E7" s="4" t="s">
-        <v>240</v>
-      </c>
-      <c r="F7" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="G7" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="H7" s="5" t="s">
-        <v>87</v>
-      </c>
-      <c r="I7" s="5" t="s">
-        <v>87</v>
-      </c>
-      <c r="J7" s="5" t="s">
-        <v>86</v>
-      </c>
-      <c r="K7" s="5" t="s">
-        <v>86</v>
-      </c>
-      <c r="L7" s="5" t="s">
-        <v>86</v>
-      </c>
-      <c r="M7" s="5" t="s">
-        <v>87</v>
-      </c>
-      <c r="N7" s="5" t="s">
-        <v>86</v>
-      </c>
-      <c r="O7" s="5" t="s">
-        <v>86</v>
-      </c>
-      <c r="P7" s="5" t="s">
-        <v>86</v>
-      </c>
-      <c r="S7" s="4" t="s">
-        <v>246</v>
-      </c>
-    </row>
-    <row r="8" spans="1:19" ht="16" x14ac:dyDescent="0.2">
-      <c r="A8" t="s">
-        <v>247</v>
-      </c>
-      <c r="B8" t="s">
-        <v>69</v>
-      </c>
-      <c r="C8" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="D8" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="E8" s="4" t="s">
-        <v>240</v>
-      </c>
-      <c r="F8" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="G8" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="H8" s="5" t="s">
-        <v>87</v>
-      </c>
-      <c r="I8" s="5" t="s">
-        <v>87</v>
-      </c>
-      <c r="J8" s="5" t="s">
-        <v>86</v>
-      </c>
-      <c r="K8" s="5" t="s">
-        <v>86</v>
-      </c>
-      <c r="L8" s="5" t="s">
-        <v>86</v>
-      </c>
-      <c r="M8" s="5" t="s">
-        <v>86</v>
-      </c>
-      <c r="O8" s="5" t="s">
-        <v>86</v>
-      </c>
-      <c r="P8" s="5" t="s">
-        <v>87</v>
-      </c>
-      <c r="Q8" s="5" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="9" spans="1:19" ht="16" x14ac:dyDescent="0.2">
-      <c r="A9" t="s">
-        <v>248</v>
-      </c>
-      <c r="B9" t="s">
-        <v>69</v>
-      </c>
-      <c r="C9" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="D9" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="E9" s="4" t="s">
-        <v>240</v>
-      </c>
-      <c r="F9" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="G9" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="H9" s="5" t="s">
-        <v>87</v>
-      </c>
-      <c r="I9" s="5" t="s">
-        <v>87</v>
-      </c>
-      <c r="J9" s="5" t="s">
-        <v>86</v>
-      </c>
-      <c r="K9" s="5" t="s">
-        <v>86</v>
-      </c>
-      <c r="L9" s="5" t="s">
-        <v>86</v>
-      </c>
-      <c r="M9" s="5" t="s">
-        <v>86</v>
-      </c>
-      <c r="O9" s="5" t="s">
-        <v>86</v>
-      </c>
-      <c r="P9" s="5" t="s">
-        <v>87</v>
-      </c>
-      <c r="Q9" s="5" t="s">
-        <v>86</v>
-      </c>
-      <c r="R9" s="5" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="10" spans="1:19" ht="32" x14ac:dyDescent="0.2">
-      <c r="A10" t="s">
-        <v>249</v>
-      </c>
-      <c r="B10" t="s">
-        <v>69</v>
-      </c>
-      <c r="C10" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="D10" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="E10" s="4" t="s">
-        <v>240</v>
-      </c>
-      <c r="F10" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="G10" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="H10" s="5" t="s">
-        <v>87</v>
-      </c>
-      <c r="I10" s="5" t="s">
-        <v>87</v>
-      </c>
-      <c r="J10" s="5" t="s">
-        <v>86</v>
-      </c>
-      <c r="K10" s="5" t="s">
-        <v>86</v>
-      </c>
-      <c r="L10" s="5" t="s">
-        <v>86</v>
-      </c>
-      <c r="M10" s="5" t="s">
-        <v>86</v>
-      </c>
-      <c r="O10" s="5" t="s">
-        <v>86</v>
-      </c>
-      <c r="P10" s="5" t="s">
-        <v>87</v>
-      </c>
-      <c r="Q10" s="5" t="s">
-        <v>86</v>
-      </c>
-      <c r="R10" s="5" t="s">
-        <v>86</v>
-      </c>
-      <c r="S10" s="4" t="s">
-        <v>250</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5EAD7908-BE00-F947-AEA2-334B464FB9B0}">
-  <dimension ref="A1:L6"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
-  <cols>
-    <col min="1" max="1" width="14.6640625" customWidth="1"/>
-    <col min="3" max="3" width="46.33203125" style="4" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="48.6640625" style="4" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="56.1640625" style="4" customWidth="1"/>
-    <col min="6" max="6" width="45.6640625" style="5" customWidth="1"/>
-    <col min="7" max="7" width="41" style="5" customWidth="1"/>
-    <col min="8" max="8" width="51.83203125" style="5" customWidth="1"/>
-    <col min="9" max="11" width="44.5" style="5" customWidth="1"/>
-    <col min="12" max="12" width="48.1640625" style="4" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:12" ht="48" x14ac:dyDescent="0.2">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="4" t="s">
-        <v>253</v>
-      </c>
-      <c r="D1" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="E1" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="F1" s="4" t="s">
-        <v>257</v>
-      </c>
-      <c r="G1" s="4" t="s">
-        <v>259</v>
-      </c>
-      <c r="H1" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="I1" s="4" t="s">
-        <v>262</v>
-      </c>
-      <c r="J1" s="4" t="s">
-        <v>264</v>
-      </c>
-      <c r="K1" s="4" t="s">
-        <v>266</v>
-      </c>
-      <c r="L1" s="4" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="2" spans="1:12" ht="16" x14ac:dyDescent="0.2">
-      <c r="A2" t="s">
-        <v>12</v>
-      </c>
-      <c r="B2" t="s">
-        <v>68</v>
-      </c>
-      <c r="C2" s="4" t="s">
-        <v>254</v>
-      </c>
-      <c r="D2" s="4" t="s">
-        <v>255</v>
-      </c>
-      <c r="E2" s="4" t="s">
-        <v>256</v>
-      </c>
-      <c r="F2" s="4" t="s">
-        <v>258</v>
-      </c>
-      <c r="G2" s="4" t="s">
-        <v>260</v>
-      </c>
-      <c r="H2" s="4" t="s">
-        <v>261</v>
-      </c>
-      <c r="I2" s="4" t="s">
-        <v>263</v>
-      </c>
-      <c r="J2" s="4" t="s">
-        <v>265</v>
-      </c>
-      <c r="K2" s="4" t="s">
-        <v>267</v>
-      </c>
-      <c r="L2" s="4" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="3" spans="1:12" ht="16" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
-        <v>251</v>
-      </c>
-      <c r="B3" t="s">
-        <v>69</v>
-      </c>
-      <c r="C3" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="D3" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="E3" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="F3" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="G3" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="H3" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="I3" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="J3" s="4" t="s">
-        <v>86</v>
-      </c>
-      <c r="K3" s="4"/>
-    </row>
-    <row r="4" spans="1:12" ht="32" x14ac:dyDescent="0.2">
-      <c r="A4" t="s">
-        <v>252</v>
-      </c>
-      <c r="B4" t="s">
-        <v>69</v>
-      </c>
-      <c r="C4" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="D4" s="4" t="s">
-        <v>86</v>
-      </c>
-      <c r="E4" s="4" t="s">
-        <v>86</v>
-      </c>
-      <c r="F4" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="G4" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="H4" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="I4" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="J4" s="4" t="s">
-        <v>86</v>
-      </c>
-      <c r="K4" s="4"/>
-      <c r="L4" s="4" t="s">
-        <v>268</v>
-      </c>
-    </row>
-    <row r="5" spans="1:12" ht="16" x14ac:dyDescent="0.2">
-      <c r="A5" t="s">
-        <v>269</v>
-      </c>
-      <c r="B5" t="s">
-        <v>69</v>
-      </c>
-      <c r="C5" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="D5" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="E5" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="F5" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="G5" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="H5" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="I5" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="J5" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="K5" s="5" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="6" spans="1:12" ht="16" x14ac:dyDescent="0.2">
-      <c r="A6" t="s">
-        <v>270</v>
-      </c>
-      <c r="B6" t="s">
-        <v>69</v>
-      </c>
-      <c r="C6" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="D6" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="E6" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="F6" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="G6" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="H6" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="I6" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="J6" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="K6" s="5" t="s">
-        <v>86</v>
-      </c>
-      <c r="L6" s="4" t="s">
-        <v>267</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{63256744-9D80-704C-8F55-50DB3E4BB623}">
-  <dimension ref="A1:J5"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
-  <cols>
-    <col min="1" max="1" width="14.6640625" customWidth="1"/>
-    <col min="3" max="3" width="46.33203125" style="4" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="48.6640625" style="4" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="56.1640625" style="4" customWidth="1"/>
-    <col min="6" max="6" width="45.6640625" style="5" customWidth="1"/>
-    <col min="7" max="7" width="41" style="5" customWidth="1"/>
-    <col min="8" max="8" width="51.83203125" style="5" customWidth="1"/>
-    <col min="9" max="9" width="44.5" style="5" customWidth="1"/>
-    <col min="10" max="10" width="48.1640625" style="4" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:10" ht="48" x14ac:dyDescent="0.2">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="4" t="s">
-        <v>289</v>
-      </c>
-      <c r="D1" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="E1" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="F1" s="4" t="s">
-        <v>257</v>
-      </c>
-      <c r="G1" s="4" t="s">
-        <v>259</v>
-      </c>
-      <c r="H1" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="I1" s="4" t="s">
-        <v>262</v>
-      </c>
-      <c r="J1" s="4" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="2" spans="1:10" ht="16" x14ac:dyDescent="0.2">
-      <c r="A2" t="s">
-        <v>12</v>
-      </c>
-      <c r="B2" t="s">
-        <v>68</v>
-      </c>
-      <c r="C2" s="4" t="s">
-        <v>290</v>
-      </c>
-      <c r="D2" s="4" t="s">
-        <v>291</v>
-      </c>
-      <c r="E2" s="4" t="s">
-        <v>292</v>
-      </c>
-      <c r="F2" s="4" t="s">
-        <v>293</v>
-      </c>
-      <c r="G2" s="4" t="s">
-        <v>294</v>
-      </c>
-      <c r="H2" s="4" t="s">
-        <v>295</v>
-      </c>
-      <c r="I2" s="4" t="s">
-        <v>296</v>
-      </c>
-      <c r="J2" s="4" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="3" spans="1:10" ht="16" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
-        <v>286</v>
-      </c>
-      <c r="B3" t="s">
-        <v>69</v>
-      </c>
-      <c r="C3" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="D3" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="E3" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="F3" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="G3" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="H3" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="I3" s="4" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="4" spans="1:10" ht="32" x14ac:dyDescent="0.2">
-      <c r="A4" t="s">
-        <v>287</v>
-      </c>
-      <c r="B4" t="s">
-        <v>69</v>
-      </c>
-      <c r="C4" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="D4" s="4" t="s">
-        <v>86</v>
-      </c>
-      <c r="E4" s="4" t="s">
-        <v>86</v>
-      </c>
-      <c r="F4" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="G4" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="H4" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="I4" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="J4" s="4" t="s">
-        <v>297</v>
-      </c>
-    </row>
-    <row r="5" spans="1:10" ht="16" x14ac:dyDescent="0.2">
-      <c r="A5" t="s">
-        <v>288</v>
-      </c>
-      <c r="B5" t="s">
-        <v>69</v>
-      </c>
-      <c r="C5" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="D5" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="E5" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="F5" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="G5" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="H5" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="I5" s="4" t="s">
-        <v>87</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E7B9AB30-85CE-ED41-92FF-29A2341C2347}">
-  <dimension ref="A1:L6"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
-  <cols>
-    <col min="1" max="1" width="14.6640625" customWidth="1"/>
-    <col min="3" max="3" width="46.33203125" style="4" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="48.6640625" style="4" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="56.1640625" style="4" customWidth="1"/>
-    <col min="6" max="6" width="45.6640625" style="5" customWidth="1"/>
-    <col min="7" max="7" width="41" style="5" customWidth="1"/>
-    <col min="8" max="8" width="51.83203125" style="5" customWidth="1"/>
-    <col min="9" max="11" width="44.5" style="5" customWidth="1"/>
-    <col min="12" max="12" width="48.1640625" style="4" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:12" ht="48" x14ac:dyDescent="0.2">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="4" t="s">
-        <v>275</v>
-      </c>
-      <c r="D1" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="E1" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="F1" s="4" t="s">
-        <v>257</v>
-      </c>
-      <c r="G1" s="4" t="s">
-        <v>259</v>
-      </c>
-      <c r="H1" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="I1" s="4" t="s">
-        <v>262</v>
-      </c>
-      <c r="J1" s="4" t="s">
-        <v>264</v>
-      </c>
-      <c r="K1" s="4" t="s">
-        <v>266</v>
-      </c>
-      <c r="L1" s="4" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="2" spans="1:12" ht="16" x14ac:dyDescent="0.2">
-      <c r="A2" t="s">
-        <v>12</v>
-      </c>
-      <c r="B2" t="s">
-        <v>68</v>
-      </c>
-      <c r="C2" s="4" t="s">
-        <v>276</v>
-      </c>
-      <c r="D2" s="4" t="s">
-        <v>277</v>
-      </c>
-      <c r="E2" s="4" t="s">
-        <v>278</v>
-      </c>
-      <c r="F2" s="4" t="s">
-        <v>279</v>
-      </c>
-      <c r="G2" s="4" t="s">
-        <v>280</v>
-      </c>
-      <c r="H2" s="4" t="s">
-        <v>281</v>
-      </c>
-      <c r="I2" s="4" t="s">
-        <v>282</v>
-      </c>
-      <c r="J2" s="4" t="s">
-        <v>283</v>
-      </c>
-      <c r="K2" s="4" t="s">
-        <v>284</v>
-      </c>
-      <c r="L2" s="4" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="3" spans="1:12" ht="16" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
-        <v>271</v>
-      </c>
-      <c r="B3" t="s">
-        <v>69</v>
-      </c>
-      <c r="C3" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="D3" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="E3" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="F3" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="G3" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="H3" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="I3" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="J3" s="4" t="s">
-        <v>86</v>
-      </c>
-      <c r="K3" s="4"/>
-    </row>
-    <row r="4" spans="1:12" ht="32" x14ac:dyDescent="0.2">
-      <c r="A4" t="s">
-        <v>272</v>
-      </c>
-      <c r="B4" t="s">
-        <v>69</v>
-      </c>
-      <c r="C4" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="D4" s="4" t="s">
-        <v>86</v>
-      </c>
-      <c r="E4" s="4" t="s">
-        <v>86</v>
-      </c>
-      <c r="F4" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="G4" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="H4" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="I4" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="J4" s="4" t="s">
-        <v>86</v>
-      </c>
-      <c r="K4" s="4"/>
-      <c r="L4" s="4" t="s">
-        <v>285</v>
-      </c>
-    </row>
-    <row r="5" spans="1:12" ht="16" x14ac:dyDescent="0.2">
-      <c r="A5" t="s">
-        <v>273</v>
-      </c>
-      <c r="B5" t="s">
-        <v>69</v>
-      </c>
-      <c r="C5" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="D5" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="E5" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="F5" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="G5" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="H5" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="I5" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="J5" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="K5" s="5" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="6" spans="1:12" ht="16" x14ac:dyDescent="0.2">
-      <c r="A6" t="s">
-        <v>274</v>
-      </c>
-      <c r="B6" t="s">
-        <v>69</v>
-      </c>
-      <c r="C6" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="D6" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="E6" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="F6" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="G6" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="H6" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="I6" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="J6" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="K6" s="5" t="s">
-        <v>86</v>
-      </c>
-      <c r="L6" s="4" t="s">
-        <v>284</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{36A5914B-A927-9D45-902A-588DFA03FD5B}">
-  <dimension ref="A1:L5"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
-  <cols>
-    <col min="1" max="1" width="14.6640625" customWidth="1"/>
-    <col min="3" max="3" width="46.33203125" style="4" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="48.6640625" style="4" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="56.1640625" style="4" customWidth="1"/>
-    <col min="6" max="6" width="45.6640625" style="5" customWidth="1"/>
-    <col min="7" max="7" width="41" style="5" customWidth="1"/>
-    <col min="8" max="8" width="51.83203125" style="5" customWidth="1"/>
-    <col min="9" max="11" width="44.5" style="5" customWidth="1"/>
-    <col min="12" max="12" width="48.1640625" style="4" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:12" ht="48" x14ac:dyDescent="0.2">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="4" t="s">
-        <v>301</v>
-      </c>
-      <c r="D1" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="E1" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="F1" s="4" t="s">
-        <v>257</v>
-      </c>
-      <c r="G1" s="4" t="s">
-        <v>259</v>
-      </c>
-      <c r="H1" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="I1" s="4" t="s">
-        <v>262</v>
-      </c>
-      <c r="J1" s="4" t="s">
-        <v>264</v>
-      </c>
-      <c r="K1" s="4" t="s">
-        <v>266</v>
-      </c>
-      <c r="L1" s="4" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="2" spans="1:12" ht="16" x14ac:dyDescent="0.2">
-      <c r="A2" t="s">
-        <v>12</v>
-      </c>
-      <c r="B2" t="s">
-        <v>68</v>
-      </c>
-      <c r="C2" s="4" t="s">
-        <v>302</v>
-      </c>
-      <c r="D2" s="4" t="s">
-        <v>303</v>
-      </c>
-      <c r="E2" s="4" t="s">
-        <v>304</v>
-      </c>
-      <c r="F2" s="4" t="s">
-        <v>305</v>
-      </c>
-      <c r="G2" s="4" t="s">
-        <v>306</v>
-      </c>
-      <c r="H2" s="4" t="s">
-        <v>307</v>
-      </c>
-      <c r="I2" s="4" t="s">
-        <v>308</v>
-      </c>
-      <c r="J2" s="4" t="s">
-        <v>283</v>
-      </c>
-      <c r="K2" s="4" t="s">
-        <v>284</v>
-      </c>
-      <c r="L2" s="4" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="3" spans="1:12" ht="16" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
-        <v>298</v>
-      </c>
-      <c r="B3" t="s">
-        <v>69</v>
-      </c>
-      <c r="C3" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="D3" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="E3" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="F3" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="G3" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="H3" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="I3" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="J3" s="4" t="s">
-        <v>86</v>
-      </c>
-      <c r="K3" s="4"/>
-    </row>
-    <row r="4" spans="1:12" ht="32" x14ac:dyDescent="0.2">
-      <c r="A4" t="s">
-        <v>299</v>
-      </c>
-      <c r="B4" t="s">
-        <v>69</v>
-      </c>
-      <c r="C4" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="D4" s="4" t="s">
-        <v>86</v>
-      </c>
-      <c r="E4" s="4" t="s">
-        <v>86</v>
-      </c>
-      <c r="F4" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="G4" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="H4" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="I4" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="J4" s="4" t="s">
-        <v>86</v>
-      </c>
-      <c r="K4" s="4"/>
-      <c r="L4" s="4" t="s">
-        <v>309</v>
-      </c>
-    </row>
-    <row r="5" spans="1:12" ht="16" x14ac:dyDescent="0.2">
-      <c r="A5" t="s">
-        <v>300</v>
-      </c>
-      <c r="B5" t="s">
-        <v>69</v>
-      </c>
-      <c r="C5" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="D5" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="E5" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="F5" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="G5" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="H5" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="I5" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="J5" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="K5" s="5" t="s">
-        <v>87</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BDE3D036-FEBF-5D43-AC42-09E358779E0F}">
-  <dimension ref="A1:K4"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
-  <cols>
-    <col min="1" max="1" width="14.6640625" customWidth="1"/>
-    <col min="3" max="3" width="46.33203125" style="4" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="48.6640625" style="4" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="56.1640625" style="4" customWidth="1"/>
-    <col min="6" max="6" width="45.6640625" style="5" customWidth="1"/>
-    <col min="7" max="7" width="41" style="5" customWidth="1"/>
-    <col min="8" max="8" width="51.83203125" style="5" customWidth="1"/>
-    <col min="9" max="9" width="44.5" style="5" customWidth="1"/>
-    <col min="10" max="10" width="39.6640625" style="5" customWidth="1"/>
-    <col min="11" max="11" width="48.1640625" style="4" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:11" ht="48" x14ac:dyDescent="0.2">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="D1" s="4" t="s">
-        <v>152</v>
-      </c>
-      <c r="E1" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="F1" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="G1" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="H1" s="4" t="s">
-        <v>157</v>
-      </c>
-      <c r="I1" s="4" t="s">
-        <v>159</v>
-      </c>
-      <c r="J1" s="4" t="s">
-        <v>160</v>
-      </c>
-      <c r="K1" s="4" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="2" spans="1:11" ht="16" x14ac:dyDescent="0.2">
-      <c r="A2" t="s">
-        <v>12</v>
-      </c>
-      <c r="B2" t="s">
-        <v>68</v>
-      </c>
-      <c r="C2" s="4" t="s">
-        <v>150</v>
-      </c>
-      <c r="D2" s="4" t="s">
-        <v>151</v>
-      </c>
-      <c r="E2" s="4" t="s">
-        <v>153</v>
-      </c>
-      <c r="F2" s="4" t="s">
-        <v>154</v>
-      </c>
-      <c r="G2" s="4" t="s">
-        <v>155</v>
-      </c>
-      <c r="H2" s="4" t="s">
-        <v>156</v>
-      </c>
-      <c r="I2" s="4" t="s">
-        <v>158</v>
-      </c>
-      <c r="J2" s="4" t="s">
-        <v>161</v>
-      </c>
-      <c r="K2" s="4" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="3" spans="1:11" ht="16" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
-        <v>162</v>
-      </c>
-      <c r="B3" t="s">
-        <v>69</v>
-      </c>
-      <c r="C3" s="4" t="s">
-        <v>77</v>
-      </c>
-      <c r="D3" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="E3" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="F3" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="G3" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="H3" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="I3" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="J3" s="4" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="4" spans="1:11" ht="32" x14ac:dyDescent="0.2">
-      <c r="A4" t="s">
-        <v>163</v>
-      </c>
-      <c r="B4" t="s">
-        <v>69</v>
-      </c>
-      <c r="C4" s="4" t="s">
-        <v>77</v>
-      </c>
-      <c r="D4" s="4" t="s">
-        <v>86</v>
-      </c>
-      <c r="E4" s="4" t="s">
-        <v>86</v>
-      </c>
-      <c r="F4" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="G4" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="H4" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="I4" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="J4" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="K4" s="4" t="s">
-        <v>164</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BE7981E0-7582-47E2-8222-6AD74E67DB3E}">
   <sheetPr>
     <tabColor rgb="FFFFFFFF"/>
@@ -3575,6 +1810,1371 @@
         <v>87</v>
       </c>
       <c r="O6" s="6"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BDE3D036-FEBF-5D43-AC42-09E358779E0F}">
+  <dimension ref="A1:K4"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="14.6640625" customWidth="1"/>
+    <col min="3" max="3" width="46.33203125" style="4" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="48.6640625" style="4" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="56.1640625" style="4" customWidth="1"/>
+    <col min="6" max="6" width="45.6640625" style="5" customWidth="1"/>
+    <col min="7" max="7" width="41" style="5" customWidth="1"/>
+    <col min="8" max="8" width="51.83203125" style="5" customWidth="1"/>
+    <col min="9" max="9" width="44.5" style="5" customWidth="1"/>
+    <col min="10" max="10" width="39.6640625" style="5" customWidth="1"/>
+    <col min="11" max="11" width="48.1640625" style="4" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:11" ht="48" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1" s="4" t="s">
+        <v>152</v>
+      </c>
+      <c r="E1" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="F1" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="G1" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1" s="4" t="s">
+        <v>157</v>
+      </c>
+      <c r="I1" s="4" t="s">
+        <v>159</v>
+      </c>
+      <c r="J1" s="4" t="s">
+        <v>160</v>
+      </c>
+      <c r="K1" s="4" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" ht="16" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B2" t="s">
+        <v>68</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>150</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>151</v>
+      </c>
+      <c r="E2" s="4" t="s">
+        <v>153</v>
+      </c>
+      <c r="F2" s="4" t="s">
+        <v>154</v>
+      </c>
+      <c r="G2" s="4" t="s">
+        <v>155</v>
+      </c>
+      <c r="H2" s="4" t="s">
+        <v>156</v>
+      </c>
+      <c r="I2" s="4" t="s">
+        <v>158</v>
+      </c>
+      <c r="J2" s="4" t="s">
+        <v>161</v>
+      </c>
+      <c r="K2" s="4" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" ht="16" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>162</v>
+      </c>
+      <c r="B3" t="s">
+        <v>69</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="F3" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="G3" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="H3" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="I3" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="J3" s="4" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" ht="32" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>163</v>
+      </c>
+      <c r="B4" t="s">
+        <v>69</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="F4" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="G4" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="H4" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="I4" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="J4" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="K4" s="4" t="s">
+        <v>164</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2B45B736-35F4-404E-994E-F08E1074E335}">
+  <dimension ref="A1:J4"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="14.6640625" customWidth="1"/>
+    <col min="3" max="3" width="46.33203125" style="4" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="48.6640625" style="4" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="56.1640625" style="4" customWidth="1"/>
+    <col min="6" max="6" width="45.6640625" style="5" customWidth="1"/>
+    <col min="7" max="7" width="41" style="5" customWidth="1"/>
+    <col min="8" max="8" width="51.83203125" style="5" customWidth="1"/>
+    <col min="9" max="9" width="44.5" style="5" customWidth="1"/>
+    <col min="10" max="10" width="48.1640625" style="4" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:10" ht="48" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>167</v>
+      </c>
+      <c r="D1" s="4" t="s">
+        <v>169</v>
+      </c>
+      <c r="E1" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="F1" s="4" t="s">
+        <v>172</v>
+      </c>
+      <c r="G1" s="4" t="s">
+        <v>174</v>
+      </c>
+      <c r="H1" s="4" t="s">
+        <v>176</v>
+      </c>
+      <c r="I1" s="4" t="s">
+        <v>178</v>
+      </c>
+      <c r="J1" s="4" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B2" t="s">
+        <v>68</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>168</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>170</v>
+      </c>
+      <c r="E2" s="4" t="s">
+        <v>171</v>
+      </c>
+      <c r="F2" s="4" t="s">
+        <v>173</v>
+      </c>
+      <c r="G2" s="4" t="s">
+        <v>175</v>
+      </c>
+      <c r="H2" s="4" t="s">
+        <v>177</v>
+      </c>
+      <c r="I2" s="4" t="s">
+        <v>179</v>
+      </c>
+      <c r="J2" s="4" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>165</v>
+      </c>
+      <c r="B3" t="s">
+        <v>69</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="F3" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="G3" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="H3" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="I3" s="4" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" ht="32" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>166</v>
+      </c>
+      <c r="B4" t="s">
+        <v>69</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="F4" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="G4" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="H4" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="I4" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="J4" s="4" t="s">
+        <v>180</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5EAD7908-BE00-F947-AEA2-334B464FB9B0}">
+  <dimension ref="A1:L6"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="14.6640625" customWidth="1"/>
+    <col min="3" max="3" width="46.33203125" style="4" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="48.6640625" style="4" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="56.1640625" style="4" customWidth="1"/>
+    <col min="6" max="6" width="45.6640625" style="5" customWidth="1"/>
+    <col min="7" max="7" width="41" style="5" customWidth="1"/>
+    <col min="8" max="8" width="51.83203125" style="5" customWidth="1"/>
+    <col min="9" max="11" width="44.5" style="5" customWidth="1"/>
+    <col min="12" max="12" width="48.1640625" style="4" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:12" ht="48" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>253</v>
+      </c>
+      <c r="D1" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="E1" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" s="4" t="s">
+        <v>257</v>
+      </c>
+      <c r="G1" s="4" t="s">
+        <v>259</v>
+      </c>
+      <c r="H1" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="I1" s="4" t="s">
+        <v>262</v>
+      </c>
+      <c r="J1" s="4" t="s">
+        <v>264</v>
+      </c>
+      <c r="K1" s="4" t="s">
+        <v>266</v>
+      </c>
+      <c r="L1" s="4" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12" ht="16" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B2" t="s">
+        <v>68</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>254</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>255</v>
+      </c>
+      <c r="E2" s="4" t="s">
+        <v>256</v>
+      </c>
+      <c r="F2" s="4" t="s">
+        <v>258</v>
+      </c>
+      <c r="G2" s="4" t="s">
+        <v>260</v>
+      </c>
+      <c r="H2" s="4" t="s">
+        <v>261</v>
+      </c>
+      <c r="I2" s="4" t="s">
+        <v>263</v>
+      </c>
+      <c r="J2" s="4" t="s">
+        <v>265</v>
+      </c>
+      <c r="K2" s="4" t="s">
+        <v>267</v>
+      </c>
+      <c r="L2" s="4" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" ht="16" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>251</v>
+      </c>
+      <c r="B3" t="s">
+        <v>69</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="F3" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="G3" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="H3" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="I3" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="J3" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="K3" s="4"/>
+    </row>
+    <row r="4" spans="1:12" ht="32" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>252</v>
+      </c>
+      <c r="B4" t="s">
+        <v>69</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="F4" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="G4" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="H4" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="I4" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="J4" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="K4" s="4"/>
+      <c r="L4" s="4" t="s">
+        <v>268</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" ht="16" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>269</v>
+      </c>
+      <c r="B5" t="s">
+        <v>69</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="E5" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="F5" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="G5" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="H5" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="I5" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="J5" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="K5" s="5" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" ht="16" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
+        <v>270</v>
+      </c>
+      <c r="B6" t="s">
+        <v>69</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="E6" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="F6" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="G6" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="H6" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="I6" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="J6" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="K6" s="5" t="s">
+        <v>86</v>
+      </c>
+      <c r="L6" s="4" t="s">
+        <v>267</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{63256744-9D80-704C-8F55-50DB3E4BB623}">
+  <dimension ref="A1:J5"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="14.6640625" customWidth="1"/>
+    <col min="3" max="3" width="46.33203125" style="4" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="48.6640625" style="4" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="56.1640625" style="4" customWidth="1"/>
+    <col min="6" max="6" width="45.6640625" style="5" customWidth="1"/>
+    <col min="7" max="7" width="41" style="5" customWidth="1"/>
+    <col min="8" max="8" width="51.83203125" style="5" customWidth="1"/>
+    <col min="9" max="9" width="44.5" style="5" customWidth="1"/>
+    <col min="10" max="10" width="48.1640625" style="4" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:10" ht="48" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>289</v>
+      </c>
+      <c r="D1" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="E1" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" s="4" t="s">
+        <v>257</v>
+      </c>
+      <c r="G1" s="4" t="s">
+        <v>259</v>
+      </c>
+      <c r="H1" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="I1" s="4" t="s">
+        <v>262</v>
+      </c>
+      <c r="J1" s="4" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B2" t="s">
+        <v>68</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>290</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>291</v>
+      </c>
+      <c r="E2" s="4" t="s">
+        <v>292</v>
+      </c>
+      <c r="F2" s="4" t="s">
+        <v>293</v>
+      </c>
+      <c r="G2" s="4" t="s">
+        <v>294</v>
+      </c>
+      <c r="H2" s="4" t="s">
+        <v>295</v>
+      </c>
+      <c r="I2" s="4" t="s">
+        <v>296</v>
+      </c>
+      <c r="J2" s="4" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>286</v>
+      </c>
+      <c r="B3" t="s">
+        <v>69</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="F3" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="G3" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="H3" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="I3" s="4" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" ht="32" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>287</v>
+      </c>
+      <c r="B4" t="s">
+        <v>69</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="F4" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="G4" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="H4" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="I4" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="J4" s="4" t="s">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>288</v>
+      </c>
+      <c r="B5" t="s">
+        <v>69</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="E5" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="F5" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="G5" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="H5" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="I5" s="4" t="s">
+        <v>87</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E7B9AB30-85CE-ED41-92FF-29A2341C2347}">
+  <dimension ref="A1:L6"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="14.6640625" customWidth="1"/>
+    <col min="3" max="3" width="46.33203125" style="4" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="48.6640625" style="4" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="56.1640625" style="4" customWidth="1"/>
+    <col min="6" max="6" width="45.6640625" style="5" customWidth="1"/>
+    <col min="7" max="7" width="41" style="5" customWidth="1"/>
+    <col min="8" max="8" width="51.83203125" style="5" customWidth="1"/>
+    <col min="9" max="11" width="44.5" style="5" customWidth="1"/>
+    <col min="12" max="12" width="48.1640625" style="4" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:12" ht="48" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>275</v>
+      </c>
+      <c r="D1" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="E1" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" s="4" t="s">
+        <v>257</v>
+      </c>
+      <c r="G1" s="4" t="s">
+        <v>259</v>
+      </c>
+      <c r="H1" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="I1" s="4" t="s">
+        <v>262</v>
+      </c>
+      <c r="J1" s="4" t="s">
+        <v>264</v>
+      </c>
+      <c r="K1" s="4" t="s">
+        <v>266</v>
+      </c>
+      <c r="L1" s="4" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12" ht="16" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B2" t="s">
+        <v>68</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>276</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>277</v>
+      </c>
+      <c r="E2" s="4" t="s">
+        <v>278</v>
+      </c>
+      <c r="F2" s="4" t="s">
+        <v>279</v>
+      </c>
+      <c r="G2" s="4" t="s">
+        <v>280</v>
+      </c>
+      <c r="H2" s="4" t="s">
+        <v>281</v>
+      </c>
+      <c r="I2" s="4" t="s">
+        <v>282</v>
+      </c>
+      <c r="J2" s="4" t="s">
+        <v>283</v>
+      </c>
+      <c r="K2" s="4" t="s">
+        <v>284</v>
+      </c>
+      <c r="L2" s="4" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" ht="16" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>271</v>
+      </c>
+      <c r="B3" t="s">
+        <v>69</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="F3" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="G3" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="H3" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="I3" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="J3" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="K3" s="4"/>
+    </row>
+    <row r="4" spans="1:12" ht="32" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>272</v>
+      </c>
+      <c r="B4" t="s">
+        <v>69</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="F4" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="G4" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="H4" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="I4" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="J4" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="K4" s="4"/>
+      <c r="L4" s="4" t="s">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" ht="16" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>273</v>
+      </c>
+      <c r="B5" t="s">
+        <v>69</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="E5" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="F5" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="G5" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="H5" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="I5" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="J5" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="K5" s="5" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" ht="16" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
+        <v>274</v>
+      </c>
+      <c r="B6" t="s">
+        <v>69</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="E6" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="F6" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="G6" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="H6" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="I6" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="J6" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="K6" s="5" t="s">
+        <v>86</v>
+      </c>
+      <c r="L6" s="4" t="s">
+        <v>284</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{36A5914B-A927-9D45-902A-588DFA03FD5B}">
+  <dimension ref="A1:L5"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="14.6640625" customWidth="1"/>
+    <col min="3" max="3" width="46.33203125" style="4" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="48.6640625" style="4" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="56.1640625" style="4" customWidth="1"/>
+    <col min="6" max="6" width="45.6640625" style="5" customWidth="1"/>
+    <col min="7" max="7" width="41" style="5" customWidth="1"/>
+    <col min="8" max="8" width="51.83203125" style="5" customWidth="1"/>
+    <col min="9" max="11" width="44.5" style="5" customWidth="1"/>
+    <col min="12" max="12" width="48.1640625" style="4" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:12" ht="48" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>301</v>
+      </c>
+      <c r="D1" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="E1" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" s="4" t="s">
+        <v>257</v>
+      </c>
+      <c r="G1" s="4" t="s">
+        <v>259</v>
+      </c>
+      <c r="H1" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="I1" s="4" t="s">
+        <v>262</v>
+      </c>
+      <c r="J1" s="4" t="s">
+        <v>264</v>
+      </c>
+      <c r="K1" s="4" t="s">
+        <v>266</v>
+      </c>
+      <c r="L1" s="4" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12" ht="16" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B2" t="s">
+        <v>68</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>302</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>303</v>
+      </c>
+      <c r="E2" s="4" t="s">
+        <v>304</v>
+      </c>
+      <c r="F2" s="4" t="s">
+        <v>305</v>
+      </c>
+      <c r="G2" s="4" t="s">
+        <v>306</v>
+      </c>
+      <c r="H2" s="4" t="s">
+        <v>307</v>
+      </c>
+      <c r="I2" s="4" t="s">
+        <v>308</v>
+      </c>
+      <c r="J2" s="4" t="s">
+        <v>283</v>
+      </c>
+      <c r="K2" s="4" t="s">
+        <v>284</v>
+      </c>
+      <c r="L2" s="4" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" ht="16" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>298</v>
+      </c>
+      <c r="B3" t="s">
+        <v>69</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="F3" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="G3" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="H3" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="I3" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="J3" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="K3" s="4"/>
+    </row>
+    <row r="4" spans="1:12" ht="32" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>299</v>
+      </c>
+      <c r="B4" t="s">
+        <v>69</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="F4" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="G4" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="H4" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="I4" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="J4" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="K4" s="4"/>
+      <c r="L4" s="4" t="s">
+        <v>309</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" ht="16" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>300</v>
+      </c>
+      <c r="B5" t="s">
+        <v>69</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="E5" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="F5" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="G5" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="H5" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="I5" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="J5" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="K5" s="5" t="s">
+        <v>87</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{521E381E-94A1-CA4C-9D15-5BDDF952F7C7}">
+  <dimension ref="A1:O4"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="14.6640625" customWidth="1"/>
+    <col min="3" max="3" width="46.33203125" style="4" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="48.6640625" style="4" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="56.1640625" style="4" customWidth="1"/>
+    <col min="6" max="6" width="45.6640625" style="5" customWidth="1"/>
+    <col min="7" max="7" width="41" style="5" customWidth="1"/>
+    <col min="8" max="8" width="51.83203125" style="5" customWidth="1"/>
+    <col min="9" max="14" width="44.5" style="5" customWidth="1"/>
+    <col min="15" max="15" width="48.1640625" style="4" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:15" ht="48" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>183</v>
+      </c>
+      <c r="D1" s="4" t="s">
+        <v>185</v>
+      </c>
+      <c r="E1" s="4" t="s">
+        <v>187</v>
+      </c>
+      <c r="F1" s="4" t="s">
+        <v>189</v>
+      </c>
+      <c r="G1" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="H1" s="4" t="s">
+        <v>192</v>
+      </c>
+      <c r="I1" s="4" t="s">
+        <v>194</v>
+      </c>
+      <c r="J1" s="4" t="s">
+        <v>196</v>
+      </c>
+      <c r="K1" s="4" t="s">
+        <v>198</v>
+      </c>
+      <c r="L1" s="4" t="s">
+        <v>200</v>
+      </c>
+      <c r="M1" s="4" t="s">
+        <v>202</v>
+      </c>
+      <c r="N1" s="4" t="s">
+        <v>204</v>
+      </c>
+      <c r="O1" s="4" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="2" spans="1:15" ht="32" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B2" t="s">
+        <v>68</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>184</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>186</v>
+      </c>
+      <c r="E2" s="4" t="s">
+        <v>188</v>
+      </c>
+      <c r="F2" s="4" t="s">
+        <v>190</v>
+      </c>
+      <c r="G2" s="4" t="s">
+        <v>191</v>
+      </c>
+      <c r="H2" s="4" t="s">
+        <v>193</v>
+      </c>
+      <c r="I2" s="4" t="s">
+        <v>195</v>
+      </c>
+      <c r="J2" s="4" t="s">
+        <v>197</v>
+      </c>
+      <c r="K2" s="4" t="s">
+        <v>199</v>
+      </c>
+      <c r="L2" s="4" t="s">
+        <v>201</v>
+      </c>
+      <c r="M2" s="4" t="s">
+        <v>203</v>
+      </c>
+      <c r="N2" s="4" t="s">
+        <v>205</v>
+      </c>
+      <c r="O2" s="4" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="3" spans="1:15" ht="16" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>181</v>
+      </c>
+      <c r="B3" t="s">
+        <v>69</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="F3" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="G3" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="H3" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="I3" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="J3" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="K3" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="L3" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="M3" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="N3" s="4" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="4" spans="1:15" ht="32" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>182</v>
+      </c>
+      <c r="B4" t="s">
+        <v>69</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="F4" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="G4" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="H4" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="I4" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="J4" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="K4" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="L4" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="M4" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="N4" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="O4" s="4" t="s">
+        <v>206</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -5707,8 +5307,8 @@
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2B45B736-35F4-404E-994E-F08E1074E335}">
-  <dimension ref="A1:J4"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{97A1D2A4-B682-FE42-B308-482711D73604}">
+  <dimension ref="A1:S10"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="14.6640625" customWidth="1"/>
@@ -5718,11 +5318,11 @@
     <col min="6" max="6" width="45.6640625" style="5" customWidth="1"/>
     <col min="7" max="7" width="41" style="5" customWidth="1"/>
     <col min="8" max="8" width="51.83203125" style="5" customWidth="1"/>
-    <col min="9" max="9" width="44.5" style="5" customWidth="1"/>
-    <col min="10" max="10" width="48.1640625" style="4" customWidth="1"/>
+    <col min="9" max="18" width="44.5" style="5" customWidth="1"/>
+    <col min="19" max="19" width="48.1640625" style="4" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="48" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:19" ht="64" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -5730,31 +5330,58 @@
         <v>1</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>167</v>
+        <v>209</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>169</v>
+        <v>211</v>
       </c>
       <c r="E1" s="4" t="s">
+        <v>213</v>
+      </c>
+      <c r="F1" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="F1" s="4" t="s">
-        <v>172</v>
-      </c>
       <c r="G1" s="4" t="s">
-        <v>174</v>
+        <v>216</v>
       </c>
       <c r="H1" s="4" t="s">
-        <v>176</v>
+        <v>218</v>
       </c>
       <c r="I1" s="4" t="s">
-        <v>178</v>
+        <v>220</v>
       </c>
       <c r="J1" s="4" t="s">
+        <v>222</v>
+      </c>
+      <c r="K1" s="4" t="s">
+        <v>224</v>
+      </c>
+      <c r="L1" s="4" t="s">
+        <v>226</v>
+      </c>
+      <c r="M1" s="4" t="s">
+        <v>228</v>
+      </c>
+      <c r="N1" s="4" t="s">
+        <v>234</v>
+      </c>
+      <c r="O1" s="4" t="s">
+        <v>230</v>
+      </c>
+      <c r="P1" s="4" t="s">
+        <v>232</v>
+      </c>
+      <c r="Q1" s="4" t="s">
+        <v>236</v>
+      </c>
+      <c r="R1" s="4" t="s">
+        <v>238</v>
+      </c>
+      <c r="S1" s="4" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="2" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:19" ht="16" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>12</v>
       </c>
@@ -5762,33 +5389,60 @@
         <v>68</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>168</v>
+        <v>210</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>170</v>
+        <v>212</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>171</v>
+        <v>214</v>
       </c>
       <c r="F2" s="4" t="s">
-        <v>173</v>
+        <v>215</v>
       </c>
       <c r="G2" s="4" t="s">
-        <v>175</v>
+        <v>217</v>
       </c>
       <c r="H2" s="4" t="s">
-        <v>177</v>
+        <v>219</v>
       </c>
       <c r="I2" s="4" t="s">
-        <v>179</v>
+        <v>221</v>
       </c>
       <c r="J2" s="4" t="s">
+        <v>223</v>
+      </c>
+      <c r="K2" s="4" t="s">
+        <v>225</v>
+      </c>
+      <c r="L2" s="4" t="s">
+        <v>227</v>
+      </c>
+      <c r="M2" s="4" t="s">
+        <v>229</v>
+      </c>
+      <c r="N2" s="4" t="s">
+        <v>235</v>
+      </c>
+      <c r="O2" s="4" t="s">
+        <v>231</v>
+      </c>
+      <c r="P2" s="4" t="s">
+        <v>233</v>
+      </c>
+      <c r="Q2" s="4" t="s">
+        <v>237</v>
+      </c>
+      <c r="R2" s="4" t="s">
+        <v>239</v>
+      </c>
+      <c r="S2" s="4" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="3" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:19" ht="16" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>165</v>
+        <v>207</v>
       </c>
       <c r="B3" t="s">
         <v>69</v>
@@ -5800,7 +5454,7 @@
         <v>87</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>87</v>
+        <v>240</v>
       </c>
       <c r="F3" s="4" t="s">
         <v>87</v>
@@ -5814,22 +5468,43 @@
       <c r="I3" s="4" t="s">
         <v>87</v>
       </c>
-    </row>
-    <row r="4" spans="1:10" ht="32" x14ac:dyDescent="0.2">
+      <c r="J3" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="K3" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="L3" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="M3" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="N3" s="4"/>
+      <c r="O3" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="P3" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="Q3" s="4"/>
+      <c r="R3" s="4"/>
+    </row>
+    <row r="4" spans="1:19" ht="32" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>166</v>
+        <v>208</v>
       </c>
       <c r="B4" t="s">
         <v>69</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="D4" s="4" t="s">
         <v>86</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>86</v>
+        <v>240</v>
       </c>
       <c r="F4" s="4" t="s">
         <v>87</v>
@@ -5844,7 +5519,332 @@
         <v>87</v>
       </c>
       <c r="J4" s="4" t="s">
-        <v>180</v>
+        <v>86</v>
+      </c>
+      <c r="K4" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="L4" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="M4" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="N4" s="4"/>
+      <c r="O4" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="P4" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="Q4" s="4"/>
+      <c r="R4" s="4"/>
+      <c r="S4" s="4" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="5" spans="1:19" ht="16" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>242</v>
+      </c>
+      <c r="B5" t="s">
+        <v>69</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="E5" s="4" t="s">
+        <v>240</v>
+      </c>
+      <c r="F5" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="G5" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="H5" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="I5" s="4"/>
+      <c r="K5" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="L5" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="M5" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="O5" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="P5" s="5" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="6" spans="1:19" ht="32" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
+        <v>243</v>
+      </c>
+      <c r="B6" t="s">
+        <v>69</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="E6" s="4" t="s">
+        <v>240</v>
+      </c>
+      <c r="F6" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="G6" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="H6" s="5" t="s">
+        <v>87</v>
+      </c>
+      <c r="I6" s="5" t="s">
+        <v>86</v>
+      </c>
+      <c r="J6" s="5" t="s">
+        <v>87</v>
+      </c>
+      <c r="K6" s="5" t="s">
+        <v>86</v>
+      </c>
+      <c r="L6" s="5" t="s">
+        <v>86</v>
+      </c>
+      <c r="M6" s="5" t="s">
+        <v>86</v>
+      </c>
+      <c r="O6" s="5" t="s">
+        <v>86</v>
+      </c>
+      <c r="P6" s="5" t="s">
+        <v>86</v>
+      </c>
+      <c r="S6" s="4" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="7" spans="1:19" ht="32" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
+        <v>245</v>
+      </c>
+      <c r="B7" t="s">
+        <v>69</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="D7" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="E7" s="4" t="s">
+        <v>240</v>
+      </c>
+      <c r="F7" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="G7" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="H7" s="5" t="s">
+        <v>87</v>
+      </c>
+      <c r="I7" s="5" t="s">
+        <v>87</v>
+      </c>
+      <c r="J7" s="5" t="s">
+        <v>86</v>
+      </c>
+      <c r="K7" s="5" t="s">
+        <v>86</v>
+      </c>
+      <c r="L7" s="5" t="s">
+        <v>86</v>
+      </c>
+      <c r="M7" s="5" t="s">
+        <v>87</v>
+      </c>
+      <c r="N7" s="5" t="s">
+        <v>86</v>
+      </c>
+      <c r="O7" s="5" t="s">
+        <v>86</v>
+      </c>
+      <c r="P7" s="5" t="s">
+        <v>86</v>
+      </c>
+      <c r="S7" s="4" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="8" spans="1:19" ht="16" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
+        <v>247</v>
+      </c>
+      <c r="B8" t="s">
+        <v>69</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="D8" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="E8" s="4" t="s">
+        <v>240</v>
+      </c>
+      <c r="F8" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="G8" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="H8" s="5" t="s">
+        <v>87</v>
+      </c>
+      <c r="I8" s="5" t="s">
+        <v>87</v>
+      </c>
+      <c r="J8" s="5" t="s">
+        <v>86</v>
+      </c>
+      <c r="K8" s="5" t="s">
+        <v>86</v>
+      </c>
+      <c r="L8" s="5" t="s">
+        <v>86</v>
+      </c>
+      <c r="M8" s="5" t="s">
+        <v>86</v>
+      </c>
+      <c r="O8" s="5" t="s">
+        <v>86</v>
+      </c>
+      <c r="P8" s="5" t="s">
+        <v>87</v>
+      </c>
+      <c r="Q8" s="5" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="9" spans="1:19" ht="16" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
+        <v>248</v>
+      </c>
+      <c r="B9" t="s">
+        <v>69</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="D9" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="E9" s="4" t="s">
+        <v>240</v>
+      </c>
+      <c r="F9" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="G9" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="H9" s="5" t="s">
+        <v>87</v>
+      </c>
+      <c r="I9" s="5" t="s">
+        <v>87</v>
+      </c>
+      <c r="J9" s="5" t="s">
+        <v>86</v>
+      </c>
+      <c r="K9" s="5" t="s">
+        <v>86</v>
+      </c>
+      <c r="L9" s="5" t="s">
+        <v>86</v>
+      </c>
+      <c r="M9" s="5" t="s">
+        <v>86</v>
+      </c>
+      <c r="O9" s="5" t="s">
+        <v>86</v>
+      </c>
+      <c r="P9" s="5" t="s">
+        <v>87</v>
+      </c>
+      <c r="Q9" s="5" t="s">
+        <v>86</v>
+      </c>
+      <c r="R9" s="5" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="10" spans="1:19" ht="32" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
+        <v>249</v>
+      </c>
+      <c r="B10" t="s">
+        <v>69</v>
+      </c>
+      <c r="C10" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="D10" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="E10" s="4" t="s">
+        <v>240</v>
+      </c>
+      <c r="F10" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="G10" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="H10" s="5" t="s">
+        <v>87</v>
+      </c>
+      <c r="I10" s="5" t="s">
+        <v>87</v>
+      </c>
+      <c r="J10" s="5" t="s">
+        <v>86</v>
+      </c>
+      <c r="K10" s="5" t="s">
+        <v>86</v>
+      </c>
+      <c r="L10" s="5" t="s">
+        <v>86</v>
+      </c>
+      <c r="M10" s="5" t="s">
+        <v>86</v>
+      </c>
+      <c r="O10" s="5" t="s">
+        <v>86</v>
+      </c>
+      <c r="P10" s="5" t="s">
+        <v>87</v>
+      </c>
+      <c r="Q10" s="5" t="s">
+        <v>86</v>
+      </c>
+      <c r="R10" s="5" t="s">
+        <v>86</v>
+      </c>
+      <c r="S10" s="4" t="s">
+        <v>250</v>
       </c>
     </row>
   </sheetData>
@@ -5853,18 +5853,12 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="ca5ba3f9-dfeb-4931-84ba-86796a0d6823">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <_ip_UnifiedCompliancePolicyUIAction xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
-    <DAte xmlns="ca5ba3f9-dfeb-4931-84ba-86796a0d6823" xsi:nil="true"/>
-    <_ip_UnifiedCompliancePolicyProperties xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
-    <date0 xmlns="ca5ba3f9-dfeb-4931-84ba-86796a0d6823" xsi:nil="true"/>
-    <TaxCatchAll xmlns="9ea08096-1d6a-4225-8886-dcb3dd04c4bd" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -6157,22 +6151,24 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="ca5ba3f9-dfeb-4931-84ba-86796a0d6823">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <_ip_UnifiedCompliancePolicyUIAction xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
+    <DAte xmlns="ca5ba3f9-dfeb-4931-84ba-86796a0d6823" xsi:nil="true"/>
+    <_ip_UnifiedCompliancePolicyProperties xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
+    <date0 xmlns="ca5ba3f9-dfeb-4931-84ba-86796a0d6823" xsi:nil="true"/>
+    <TaxCatchAll xmlns="9ea08096-1d6a-4225-8886-dcb3dd04c4bd" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3F5E14B5-D6EF-401C-82ED-6CA5F26974B2}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6A69F337-BFDC-4B9A-9645-ACD2998E51C5}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="ca5ba3f9-dfeb-4931-84ba-86796a0d6823"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
-    <ds:schemaRef ds:uri="9ea08096-1d6a-4225-8886-dcb3dd04c4bd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -6199,9 +6195,13 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6A69F337-BFDC-4B9A-9645-ACD2998E51C5}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3F5E14B5-D6EF-401C-82ED-6CA5F26974B2}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="ca5ba3f9-dfeb-4931-84ba-86796a0d6823"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
+    <ds:schemaRef ds:uri="9ea08096-1d6a-4225-8886-dcb3dd04c4bd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
[DG22-2638] Update - add dependency to test job before run build and deploy - add retry configuration for cypress
</commit_message>
<xml_diff>
--- a/packages/test/cypress/fixtures/data.xlsx
+++ b/packages/test/cypress/fixtures/data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/felix/kororo/repository/safeguard-github/rules-interface/packages/test/cypress/fixtures/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8AF1E870-CAD7-724D-98F3-19D8348E173C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F1EB216A-425E-1C44-B4B5-BF779DE202FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="19940" yWindow="500" windowWidth="18460" windowHeight="21100" tabRatio="816" firstSheet="22" activeTab="28" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="38400" windowHeight="21100" tabRatio="816" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="HVAC1_C" sheetId="1" r:id="rId1"/>
@@ -6673,7 +6673,7 @@
     <col min="18" max="16384" width="8.83203125" style="29"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" ht="64" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:17" ht="48" x14ac:dyDescent="0.2">
       <c r="A1" s="29" t="s">
         <v>0</v>
       </c>
@@ -8629,7 +8629,7 @@
     <col min="1" max="1" width="11" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="11.6640625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="12.33203125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="11.83203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="18.6640625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="15" style="6" customWidth="1"/>
     <col min="7" max="7" width="23.1640625" style="2" customWidth="1"/>
     <col min="8" max="8" width="4.6640625" bestFit="1" customWidth="1"/>
@@ -10334,12 +10334,18 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="ca5ba3f9-dfeb-4931-84ba-86796a0d6823">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <_ip_UnifiedCompliancePolicyUIAction xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
+    <DAte xmlns="ca5ba3f9-dfeb-4931-84ba-86796a0d6823" xsi:nil="true"/>
+    <_ip_UnifiedCompliancePolicyProperties xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
+    <date0 xmlns="ca5ba3f9-dfeb-4931-84ba-86796a0d6823" xsi:nil="true"/>
+    <TaxCatchAll xmlns="9ea08096-1d6a-4225-8886-dcb3dd04c4bd" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -10632,24 +10638,22 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="ca5ba3f9-dfeb-4931-84ba-86796a0d6823">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <_ip_UnifiedCompliancePolicyUIAction xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
-    <DAte xmlns="ca5ba3f9-dfeb-4931-84ba-86796a0d6823" xsi:nil="true"/>
-    <_ip_UnifiedCompliancePolicyProperties xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
-    <date0 xmlns="ca5ba3f9-dfeb-4931-84ba-86796a0d6823" xsi:nil="true"/>
-    <TaxCatchAll xmlns="9ea08096-1d6a-4225-8886-dcb3dd04c4bd" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6A69F337-BFDC-4B9A-9645-ACD2998E51C5}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3F5E14B5-D6EF-401C-82ED-6CA5F26974B2}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="ca5ba3f9-dfeb-4931-84ba-86796a0d6823"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
+    <ds:schemaRef ds:uri="9ea08096-1d6a-4225-8886-dcb3dd04c4bd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -10676,13 +10680,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3F5E14B5-D6EF-401C-82ED-6CA5F26974B2}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6A69F337-BFDC-4B9A-9645-ACD2998E51C5}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="ca5ba3f9-dfeb-4931-84ba-86796a0d6823"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
-    <ds:schemaRef ds:uri="9ea08096-1d6a-4225-8886-dcb3dd04c4bd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
[DG22-2638] try to remove loop for each test and define every test case using it in all eligibility activities
</commit_message>
<xml_diff>
--- a/packages/test/cypress/fixtures/data.xlsx
+++ b/packages/test/cypress/fixtures/data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/felix/kororo/repository/safeguard-github/rules-interface/packages/test/cypress/fixtures/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A0F5B7A5-EA5B-084B-80BD-B86C1E83F75E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6B601236-50CA-B344-9AD8-0A27181D4257}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="38400" windowHeight="21100" tabRatio="816" firstSheet="11" activeTab="21" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="38400" windowHeight="21100" tabRatio="816" firstSheet="10" activeTab="28" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="BESS2_C" sheetId="11" r:id="rId1"/>
@@ -35,9 +35,9 @@
     <sheet name="F7_C" sheetId="25" r:id="rId20"/>
     <sheet name="F7_E" sheetId="32" r:id="rId21"/>
     <sheet name="HVAC1_D16_C" sheetId="1" r:id="rId22"/>
-    <sheet name="HVAC1_E" sheetId="4" r:id="rId23"/>
-    <sheet name="HVAC2_C" sheetId="20" r:id="rId24"/>
-    <sheet name="HVAC2_E" sheetId="27" r:id="rId25"/>
+    <sheet name="HVAC1_D16_E" sheetId="4" r:id="rId23"/>
+    <sheet name="HVAC2_F4_C" sheetId="20" r:id="rId24"/>
+    <sheet name="HVAC2_F4_E" sheetId="27" r:id="rId25"/>
     <sheet name="RF2_F1_2_C" sheetId="24" r:id="rId26"/>
     <sheet name="RF2_F1_2_E" sheetId="31" r:id="rId27"/>
     <sheet name="SYS2_D5_C" sheetId="5" r:id="rId28"/>
@@ -48,7 +48,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="19" hidden="1">F7_C!$C$1:$C$8</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="21" hidden="1">HVAC1_D16_C!$D$1:$D$13</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="23" hidden="1">HVAC2_C!$D$1:$D$10</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="23" hidden="1">HVAC2_F4_C!$D$1:$D$10</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
   <extLst>
@@ -1423,72 +1423,36 @@
     <t>HVAC1_PDRSAug24_ACOP_eligible</t>
   </si>
   <si>
-    <t>HVAC1_E_001</t>
-  </si>
-  <si>
     <t>average_zone</t>
   </si>
   <si>
-    <t>HVAC1_E_002</t>
-  </si>
-  <si>
     <t>HVAC1_PDRSAug24_new_equipment_cooling_capacity,HVAC1_PDRSAug24_AEER_greater_than_minimum,HVAC1_PDRSAug24_new_equipment_heating_capacity</t>
   </si>
   <si>
-    <t>HVAC1_E_003</t>
-  </si>
-  <si>
-    <t>HVAC1_E_004</t>
-  </si>
-  <si>
     <t>HVAC2_PDRSAug24_Activity</t>
   </si>
   <si>
     <t>HVAC2_PDRSAug24_Air_Conditioner_type</t>
   </si>
   <si>
-    <t>HVAC2_C_001</t>
-  </si>
-  <si>
-    <t>HVAC2_C_002</t>
-  </si>
-  <si>
-    <t>HVAC2_C_003</t>
-  </si>
-  <si>
-    <t>HVAC2_C_004</t>
-  </si>
-  <si>
     <t>BRIVIS</t>
   </si>
   <si>
     <t>AONSR13B1-AINHU11B1</t>
   </si>
   <si>
-    <t>HVAC2_C_005</t>
-  </si>
-  <si>
     <t>DAIKIN</t>
   </si>
   <si>
     <t>REYQ16BYM</t>
   </si>
   <si>
-    <t>HVAC2_C_006</t>
-  </si>
-  <si>
-    <t>HVAC2_C_007</t>
-  </si>
-  <si>
     <t>SAMSUNG ELECTRONICS</t>
   </si>
   <si>
     <t>AM080DXVGGH-SA</t>
   </si>
   <si>
-    <t>HVAC2_C_008</t>
-  </si>
-  <si>
     <t>MITSUBISHI HEAVY INDUSTRIES</t>
   </si>
   <si>
@@ -1570,33 +1534,18 @@
     <t>HVAC2_HSPF_mixed_eligible</t>
   </si>
   <si>
-    <t>HVAC2_E_001</t>
-  </si>
-  <si>
-    <t>HVAC2_E_002</t>
-  </si>
-  <si>
     <t>HVAC2_installed_by_qualified_person,HVAC2_engaged_ACP,HVAC2_equipment_registered_in_GEMS,HVAC2_new_equipment_cooling_capacity,HVAC2_AEER_greater_than_minimum,HVAC2_new_equipment_heating_capacity,HVAC2_ACOP_eligible</t>
   </si>
   <si>
-    <t>HVAC2_E_003</t>
-  </si>
-  <si>
     <t xml:space="preserve">HVAC2_HSPF_mixed_eligible </t>
   </si>
   <si>
-    <t>HVAC2_E_004</t>
-  </si>
-  <si>
     <t>cold_zone</t>
   </si>
   <si>
     <t>HVAC2_installed_by_qualified_person,HVAC2_engaged_ACP,HVAC2_equipment_registered_in_GEMS,HVAC2_new_equipment_cooling_capacity,HVAC2_AEER_greater_than_minimum,HVAC2_HSPF_cold_eligible</t>
   </si>
   <si>
-    <t>HVAC2_E_005</t>
-  </si>
-  <si>
     <t>HVAC2_residential_building,HVAC2_installed_centralised_system_common_area_BCA_Class2_building</t>
   </si>
   <si>
@@ -1780,12 +1729,6 @@
     <t>SYS2_PDRSAug24_warranty</t>
   </si>
   <si>
-    <t>SYS2_E_001</t>
-  </si>
-  <si>
-    <t>SYS2_E_002</t>
-  </si>
-  <si>
     <t>SYS2_PDRSAug24_equipment_installed_on_site,SYS2_PDRSAug24_qualified_install_removal</t>
   </si>
   <si>
@@ -1892,6 +1835,63 @@
   </si>
   <si>
     <t>SYS2_D5_C_007</t>
+  </si>
+  <si>
+    <t>HVAC1_D16_E_001</t>
+  </si>
+  <si>
+    <t>HVAC1_D16_E_002</t>
+  </si>
+  <si>
+    <t>HVAC1_D16_E_003</t>
+  </si>
+  <si>
+    <t>HVAC1_D16_E_004</t>
+  </si>
+  <si>
+    <t>HVAC2_F4_C_001</t>
+  </si>
+  <si>
+    <t>HVAC2_F4_C_002</t>
+  </si>
+  <si>
+    <t>HVAC2_F4_C_003</t>
+  </si>
+  <si>
+    <t>HVAC2_F4_C_004</t>
+  </si>
+  <si>
+    <t>HVAC2_F4_C_005</t>
+  </si>
+  <si>
+    <t>HVAC2_F4_C_006</t>
+  </si>
+  <si>
+    <t>HVAC2_F4_C_007</t>
+  </si>
+  <si>
+    <t>HVAC2_F4_C_008</t>
+  </si>
+  <si>
+    <t>HVAC2_F4_E_001</t>
+  </si>
+  <si>
+    <t>HVAC2_F4_E_002</t>
+  </si>
+  <si>
+    <t>HVAC2_F4_E_003</t>
+  </si>
+  <si>
+    <t>HVAC2_F4_E_004</t>
+  </si>
+  <si>
+    <t>HVAC2_F4_E_005</t>
+  </si>
+  <si>
+    <t>SYS2_D5_E_001</t>
+  </si>
+  <si>
+    <t>SYS2_D5_E_002</t>
   </si>
 </sst>
 </file>
@@ -2846,10 +2846,10 @@
         <v>145</v>
       </c>
       <c r="H5" s="2">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="I5" s="2">
-        <v>41.29</v>
+        <v>37.79</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.2">
@@ -2933,10 +2933,10 @@
         <v>160</v>
       </c>
       <c r="H8">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="I8">
-        <v>21.99</v>
+        <v>18.48</v>
       </c>
     </row>
   </sheetData>
@@ -5793,7 +5793,7 @@
     </row>
     <row r="3" spans="1:11" s="11" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A3" s="10" t="s">
-        <v>589</v>
+        <v>570</v>
       </c>
       <c r="B3" s="10" t="s">
         <v>15</v>
@@ -5828,7 +5828,7 @@
     </row>
     <row r="4" spans="1:11" s="11" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A4" s="10" t="s">
-        <v>590</v>
+        <v>571</v>
       </c>
       <c r="B4" s="10" t="s">
         <v>15</v>
@@ -5863,7 +5863,7 @@
     </row>
     <row r="5" spans="1:11" s="11" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A5" s="10" t="s">
-        <v>591</v>
+        <v>572</v>
       </c>
       <c r="B5" s="10" t="s">
         <v>15</v>
@@ -5898,7 +5898,7 @@
     </row>
     <row r="6" spans="1:11" s="11" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A6" s="10" t="s">
-        <v>592</v>
+        <v>573</v>
       </c>
       <c r="B6" s="10" t="s">
         <v>15</v>
@@ -5933,7 +5933,7 @@
     </row>
     <row r="7" spans="1:11" s="11" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A7" s="10" t="s">
-        <v>593</v>
+        <v>574</v>
       </c>
       <c r="B7" s="10" t="s">
         <v>15</v>
@@ -5968,7 +5968,7 @@
     </row>
     <row r="8" spans="1:11" s="11" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A8" s="10" t="s">
-        <v>594</v>
+        <v>575</v>
       </c>
       <c r="B8" s="10" t="s">
         <v>15</v>
@@ -6003,7 +6003,7 @@
     </row>
     <row r="9" spans="1:11" s="11" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A9" s="10" t="s">
-        <v>595</v>
+        <v>576</v>
       </c>
       <c r="B9" s="10" t="s">
         <v>15</v>
@@ -6038,7 +6038,7 @@
     </row>
     <row r="10" spans="1:11" s="11" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A10" s="10" t="s">
-        <v>596</v>
+        <v>577</v>
       </c>
       <c r="B10" s="10" t="s">
         <v>15</v>
@@ -6073,7 +6073,7 @@
     </row>
     <row r="11" spans="1:11" s="11" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A11" s="10" t="s">
-        <v>597</v>
+        <v>578</v>
       </c>
       <c r="B11" s="10" t="s">
         <v>15</v>
@@ -6108,7 +6108,7 @@
     </row>
     <row r="12" spans="1:11" s="11" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A12" s="10" t="s">
-        <v>598</v>
+        <v>579</v>
       </c>
       <c r="B12" s="10" t="s">
         <v>15</v>
@@ -6143,7 +6143,7 @@
     </row>
     <row r="13" spans="1:11" s="11" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A13" s="10" t="s">
-        <v>599</v>
+        <v>580</v>
       </c>
       <c r="B13" s="10" t="s">
         <v>15</v>
@@ -6191,7 +6191,7 @@
   <dimension ref="A1:P6"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="13.83203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.33203125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="11.6640625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="52.83203125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="58.6640625" style="8" customWidth="1"/>
@@ -6308,7 +6308,7 @@
     </row>
     <row r="3" spans="1:16" ht="16" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
-        <v>450</v>
+        <v>588</v>
       </c>
       <c r="B3" s="2" t="s">
         <v>15</v>
@@ -6339,7 +6339,7 @@
       </c>
       <c r="K3" s="7"/>
       <c r="L3" s="4" t="s">
-        <v>451</v>
+        <v>450</v>
       </c>
       <c r="M3" s="7" t="s">
         <v>16</v>
@@ -6352,7 +6352,7 @@
     </row>
     <row r="4" spans="1:16" ht="48" x14ac:dyDescent="0.2">
       <c r="A4" s="2" t="s">
-        <v>452</v>
+        <v>589</v>
       </c>
       <c r="B4" s="2" t="s">
         <v>15</v>
@@ -6383,7 +6383,7 @@
         <v>55</v>
       </c>
       <c r="L4" s="4" t="s">
-        <v>451</v>
+        <v>450</v>
       </c>
       <c r="M4" s="7" t="s">
         <v>55</v>
@@ -6393,12 +6393,12 @@
         <v>16</v>
       </c>
       <c r="P4" s="3" t="s">
-        <v>453</v>
+        <v>451</v>
       </c>
     </row>
     <row r="5" spans="1:16" ht="16" x14ac:dyDescent="0.2">
       <c r="A5" s="2" t="s">
-        <v>454</v>
+        <v>590</v>
       </c>
       <c r="B5" s="2" t="s">
         <v>15</v>
@@ -6429,7 +6429,7 @@
       </c>
       <c r="K5" s="7"/>
       <c r="L5" s="4" t="s">
-        <v>451</v>
+        <v>450</v>
       </c>
       <c r="M5" s="7" t="s">
         <v>16</v>
@@ -6440,7 +6440,7 @@
     </row>
     <row r="6" spans="1:16" ht="16" x14ac:dyDescent="0.2">
       <c r="A6" s="2" t="s">
-        <v>455</v>
+        <v>591</v>
       </c>
       <c r="B6" s="2" t="s">
         <v>15</v>
@@ -6471,7 +6471,7 @@
       </c>
       <c r="K6" s="7"/>
       <c r="L6" s="4" t="s">
-        <v>451</v>
+        <v>450</v>
       </c>
       <c r="M6" s="7" t="s">
         <v>16</v>
@@ -6483,6 +6483,7 @@
       <c r="P6" s="3"/>
     </row>
   </sheetData>
+  <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -6558,10 +6559,10 @@
         <v>139</v>
       </c>
       <c r="F2" s="20" t="s">
-        <v>456</v>
+        <v>452</v>
       </c>
       <c r="G2" s="20" t="s">
-        <v>457</v>
+        <v>453</v>
       </c>
       <c r="H2" s="20" t="s">
         <v>64</v>
@@ -6578,7 +6579,7 @@
     </row>
     <row r="3" spans="1:11" ht="15.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="20" t="s">
-        <v>458</v>
+        <v>592</v>
       </c>
       <c r="B3" s="20" t="s">
         <v>15</v>
@@ -6613,7 +6614,7 @@
     </row>
     <row r="4" spans="1:11" ht="15.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="20" t="s">
-        <v>459</v>
+        <v>593</v>
       </c>
       <c r="B4" s="20" t="s">
         <v>15</v>
@@ -6648,7 +6649,7 @@
     </row>
     <row r="5" spans="1:11" ht="15.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="20" t="s">
-        <v>460</v>
+        <v>594</v>
       </c>
       <c r="B5" s="20" t="s">
         <v>15</v>
@@ -6683,7 +6684,7 @@
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A6" s="20" t="s">
-        <v>461</v>
+        <v>595</v>
       </c>
       <c r="B6" s="20" t="s">
         <v>15</v>
@@ -6692,10 +6693,10 @@
         <v>2390</v>
       </c>
       <c r="D6" s="20" t="s">
-        <v>462</v>
+        <v>454</v>
       </c>
       <c r="E6" s="20" t="s">
-        <v>463</v>
+        <v>455</v>
       </c>
       <c r="F6" s="20" t="s">
         <v>409</v>
@@ -6718,7 +6719,7 @@
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A7" s="20" t="s">
-        <v>464</v>
+        <v>596</v>
       </c>
       <c r="B7" s="20" t="s">
         <v>15</v>
@@ -6727,10 +6728,10 @@
         <v>2640</v>
       </c>
       <c r="D7" s="20" t="s">
-        <v>465</v>
+        <v>456</v>
       </c>
       <c r="E7" s="20" t="s">
-        <v>466</v>
+        <v>457</v>
       </c>
       <c r="F7" s="20" t="s">
         <v>409</v>
@@ -6753,7 +6754,7 @@
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A8" s="20" t="s">
-        <v>467</v>
+        <v>597</v>
       </c>
       <c r="B8" s="20" t="s">
         <v>15</v>
@@ -6762,10 +6763,10 @@
         <v>2222</v>
       </c>
       <c r="D8" s="20" t="s">
-        <v>465</v>
+        <v>456</v>
       </c>
       <c r="E8" s="20" t="s">
-        <v>466</v>
+        <v>457</v>
       </c>
       <c r="F8" s="20" t="s">
         <v>409</v>
@@ -6788,7 +6789,7 @@
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A9" s="20" t="s">
-        <v>468</v>
+        <v>598</v>
       </c>
       <c r="B9" s="20" t="s">
         <v>15</v>
@@ -6797,10 +6798,10 @@
         <v>2650</v>
       </c>
       <c r="D9" s="20" t="s">
-        <v>469</v>
+        <v>458</v>
       </c>
       <c r="E9" s="20" t="s">
-        <v>470</v>
+        <v>459</v>
       </c>
       <c r="F9" s="20" t="s">
         <v>405</v>
@@ -6823,7 +6824,7 @@
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A10" s="20" t="s">
-        <v>471</v>
+        <v>599</v>
       </c>
       <c r="B10" s="20" t="s">
         <v>15</v>
@@ -6832,10 +6833,10 @@
         <v>2650</v>
       </c>
       <c r="D10" s="20" t="s">
-        <v>472</v>
+        <v>460</v>
       </c>
       <c r="E10" s="20" t="s">
-        <v>473</v>
+        <v>461</v>
       </c>
       <c r="F10" s="20" t="s">
         <v>409</v>
@@ -6876,7 +6877,8 @@
   <dimension ref="A1:Q7"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="2" width="11.6640625" style="29" customWidth="1"/>
+    <col min="1" max="1" width="14.83203125" style="29" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.6640625" style="29" customWidth="1"/>
     <col min="3" max="3" width="42.1640625" style="29" customWidth="1"/>
     <col min="4" max="4" width="55.5" style="31" customWidth="1"/>
     <col min="5" max="5" width="45.5" style="31" customWidth="1"/>
@@ -6907,37 +6909,37 @@
         <v>286</v>
       </c>
       <c r="F1" s="30" t="s">
-        <v>474</v>
+        <v>462</v>
       </c>
       <c r="G1" s="30" t="s">
-        <v>475</v>
+        <v>463</v>
       </c>
       <c r="H1" s="30" t="s">
-        <v>476</v>
+        <v>464</v>
       </c>
       <c r="I1" s="30" t="s">
-        <v>477</v>
+        <v>465</v>
       </c>
       <c r="J1" s="30" t="s">
-        <v>478</v>
+        <v>466</v>
       </c>
       <c r="K1" s="30" t="s">
-        <v>479</v>
+        <v>467</v>
       </c>
       <c r="L1" s="30" t="s">
-        <v>480</v>
+        <v>468</v>
       </c>
       <c r="M1" s="30" t="s">
-        <v>481</v>
+        <v>469</v>
       </c>
       <c r="N1" s="30" t="s">
-        <v>482</v>
+        <v>470</v>
       </c>
       <c r="O1" s="30" t="s">
-        <v>483</v>
+        <v>471</v>
       </c>
       <c r="P1" s="30" t="s">
-        <v>484</v>
+        <v>472</v>
       </c>
       <c r="Q1" s="30" t="s">
         <v>39</v>
@@ -6951,46 +6953,46 @@
         <v>8</v>
       </c>
       <c r="C2" s="30" t="s">
+        <v>473</v>
+      </c>
+      <c r="D2" s="30" t="s">
+        <v>474</v>
+      </c>
+      <c r="E2" s="30" t="s">
+        <v>475</v>
+      </c>
+      <c r="F2" s="30" t="s">
+        <v>476</v>
+      </c>
+      <c r="G2" s="30" t="s">
+        <v>477</v>
+      </c>
+      <c r="H2" s="30" t="s">
+        <v>478</v>
+      </c>
+      <c r="I2" s="30" t="s">
+        <v>479</v>
+      </c>
+      <c r="J2" s="30" t="s">
+        <v>480</v>
+      </c>
+      <c r="K2" s="30" t="s">
+        <v>481</v>
+      </c>
+      <c r="L2" s="30" t="s">
+        <v>482</v>
+      </c>
+      <c r="M2" s="30" t="s">
+        <v>483</v>
+      </c>
+      <c r="N2" s="30" t="s">
+        <v>484</v>
+      </c>
+      <c r="O2" s="30" t="s">
         <v>485</v>
       </c>
-      <c r="D2" s="30" t="s">
+      <c r="P2" s="30" t="s">
         <v>486</v>
-      </c>
-      <c r="E2" s="30" t="s">
-        <v>487</v>
-      </c>
-      <c r="F2" s="30" t="s">
-        <v>488</v>
-      </c>
-      <c r="G2" s="30" t="s">
-        <v>489</v>
-      </c>
-      <c r="H2" s="30" t="s">
-        <v>490</v>
-      </c>
-      <c r="I2" s="30" t="s">
-        <v>491</v>
-      </c>
-      <c r="J2" s="30" t="s">
-        <v>492</v>
-      </c>
-      <c r="K2" s="30" t="s">
-        <v>493</v>
-      </c>
-      <c r="L2" s="30" t="s">
-        <v>494</v>
-      </c>
-      <c r="M2" s="30" t="s">
-        <v>495</v>
-      </c>
-      <c r="N2" s="30" t="s">
-        <v>496</v>
-      </c>
-      <c r="O2" s="30" t="s">
-        <v>497</v>
-      </c>
-      <c r="P2" s="30" t="s">
-        <v>498</v>
       </c>
       <c r="Q2" s="30" t="s">
         <v>52</v>
@@ -6998,7 +7000,7 @@
     </row>
     <row r="3" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A3" s="29" t="s">
-        <v>499</v>
+        <v>600</v>
       </c>
       <c r="B3" s="29" t="s">
         <v>15</v>
@@ -7027,7 +7029,7 @@
         <v>16</v>
       </c>
       <c r="L3" s="32" t="s">
-        <v>451</v>
+        <v>450</v>
       </c>
       <c r="M3" s="32" t="s">
         <v>16</v>
@@ -7040,7 +7042,7 @@
     </row>
     <row r="4" spans="1:17" ht="64" x14ac:dyDescent="0.2">
       <c r="A4" s="29" t="s">
-        <v>500</v>
+        <v>601</v>
       </c>
       <c r="B4" s="29" t="s">
         <v>15</v>
@@ -7069,7 +7071,7 @@
       </c>
       <c r="K4" s="32"/>
       <c r="L4" s="32" t="s">
-        <v>451</v>
+        <v>450</v>
       </c>
       <c r="M4" s="32" t="s">
         <v>55</v>
@@ -7080,12 +7082,12 @@
       <c r="O4" s="32"/>
       <c r="P4" s="32"/>
       <c r="Q4" s="30" t="s">
-        <v>501</v>
+        <v>487</v>
       </c>
     </row>
     <row r="5" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A5" s="29" t="s">
-        <v>502</v>
+        <v>602</v>
       </c>
       <c r="B5" s="29" t="s">
         <v>15</v>
@@ -7114,7 +7116,7 @@
         <v>16</v>
       </c>
       <c r="L5" s="32" t="s">
-        <v>451</v>
+        <v>450</v>
       </c>
       <c r="M5" s="32" t="s">
         <v>16</v>
@@ -7125,12 +7127,12 @@
         <v>55</v>
       </c>
       <c r="Q5" s="30" t="s">
-        <v>503</v>
+        <v>488</v>
       </c>
     </row>
     <row r="6" spans="1:17" ht="64" x14ac:dyDescent="0.2">
       <c r="A6" s="29" t="s">
-        <v>504</v>
+        <v>603</v>
       </c>
       <c r="B6" s="29" t="s">
         <v>15</v>
@@ -7159,7 +7161,7 @@
       </c>
       <c r="K6" s="32"/>
       <c r="L6" s="30" t="s">
-        <v>505</v>
+        <v>489</v>
       </c>
       <c r="M6" s="32" t="s">
         <v>16</v>
@@ -7170,12 +7172,12 @@
       </c>
       <c r="P6" s="32"/>
       <c r="Q6" s="30" t="s">
-        <v>506</v>
+        <v>490</v>
       </c>
     </row>
     <row r="7" spans="1:17" ht="32" x14ac:dyDescent="0.2">
       <c r="A7" s="29" t="s">
-        <v>507</v>
+        <v>604</v>
       </c>
       <c r="B7" s="29" t="s">
         <v>15</v>
@@ -7206,7 +7208,7 @@
         <v>16</v>
       </c>
       <c r="L7" s="32" t="s">
-        <v>451</v>
+        <v>450</v>
       </c>
       <c r="M7" s="32" t="s">
         <v>16</v>
@@ -7217,10 +7219,11 @@
         <v>16</v>
       </c>
       <c r="Q7" s="30" t="s">
-        <v>508</v>
+        <v>491</v>
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
@@ -7265,7 +7268,7 @@
         <v>135</v>
       </c>
       <c r="G1" s="12" t="s">
-        <v>509</v>
+        <v>492</v>
       </c>
       <c r="H1" s="12" t="s">
         <v>59</v>
@@ -7297,10 +7300,10 @@
         <v>139</v>
       </c>
       <c r="F2" s="15" t="s">
-        <v>510</v>
+        <v>493</v>
       </c>
       <c r="G2" s="15" t="s">
-        <v>511</v>
+        <v>494</v>
       </c>
       <c r="H2" s="12" t="s">
         <v>64</v>
@@ -7317,7 +7320,7 @@
     </row>
     <row r="3" spans="1:11" ht="15.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="12" t="s">
-        <v>583</v>
+        <v>564</v>
       </c>
       <c r="B3" s="12" t="s">
         <v>15</v>
@@ -7326,16 +7329,16 @@
         <v>2440</v>
       </c>
       <c r="D3" s="12" t="s">
-        <v>512</v>
+        <v>495</v>
       </c>
       <c r="E3" s="12" t="s">
-        <v>513</v>
+        <v>496</v>
       </c>
       <c r="F3" s="14" t="s">
         <v>16</v>
       </c>
       <c r="G3" s="12" t="s">
-        <v>514</v>
+        <v>497</v>
       </c>
       <c r="H3" s="12">
         <v>27</v>
@@ -7352,7 +7355,7 @@
     </row>
     <row r="4" spans="1:11" ht="15.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="12" t="s">
-        <v>584</v>
+        <v>565</v>
       </c>
       <c r="B4" s="12" t="s">
         <v>15</v>
@@ -7361,16 +7364,16 @@
         <v>2010</v>
       </c>
       <c r="D4" s="12" t="s">
-        <v>515</v>
+        <v>498</v>
       </c>
       <c r="E4" s="12" t="s">
-        <v>516</v>
+        <v>499</v>
       </c>
       <c r="F4" s="14" t="s">
         <v>55</v>
       </c>
       <c r="G4" s="12" t="s">
-        <v>517</v>
+        <v>500</v>
       </c>
       <c r="H4" s="12">
         <v>98</v>
@@ -7387,7 +7390,7 @@
     </row>
     <row r="5" spans="1:11" ht="15.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="12" t="s">
-        <v>585</v>
+        <v>566</v>
       </c>
       <c r="B5" s="12" t="s">
         <v>15</v>
@@ -7396,16 +7399,16 @@
         <v>2148</v>
       </c>
       <c r="D5" s="12" t="s">
-        <v>518</v>
+        <v>501</v>
       </c>
       <c r="E5" s="12" t="s">
-        <v>519</v>
+        <v>502</v>
       </c>
       <c r="F5" s="14" t="s">
         <v>16</v>
       </c>
       <c r="G5" s="12" t="s">
-        <v>514</v>
+        <v>497</v>
       </c>
       <c r="H5" s="12">
         <v>0</v>
@@ -7458,16 +7461,16 @@
         <v>1</v>
       </c>
       <c r="C1" s="30" t="s">
-        <v>520</v>
+        <v>503</v>
       </c>
       <c r="D1" s="30" t="s">
-        <v>521</v>
+        <v>504</v>
       </c>
       <c r="E1" s="30" t="s">
         <v>283</v>
       </c>
       <c r="F1" s="30" t="s">
-        <v>522</v>
+        <v>505</v>
       </c>
       <c r="G1" s="30" t="s">
         <v>286</v>
@@ -7476,22 +7479,22 @@
         <v>287</v>
       </c>
       <c r="I1" s="30" t="s">
-        <v>523</v>
+        <v>506</v>
       </c>
       <c r="J1" s="30" t="s">
-        <v>524</v>
+        <v>507</v>
       </c>
       <c r="K1" s="30" t="s">
-        <v>525</v>
+        <v>508</v>
       </c>
       <c r="L1" s="30" t="s">
-        <v>526</v>
+        <v>509</v>
       </c>
       <c r="M1" s="30" t="s">
-        <v>527</v>
+        <v>510</v>
       </c>
       <c r="N1" s="30" t="s">
-        <v>528</v>
+        <v>511</v>
       </c>
       <c r="O1" s="31" t="s">
         <v>39</v>
@@ -7505,40 +7508,40 @@
         <v>8</v>
       </c>
       <c r="C2" s="31" t="s">
-        <v>529</v>
+        <v>512</v>
       </c>
       <c r="D2" s="30" t="s">
-        <v>530</v>
+        <v>513</v>
       </c>
       <c r="E2" s="31" t="s">
-        <v>531</v>
+        <v>514</v>
       </c>
       <c r="F2" s="31" t="s">
-        <v>532</v>
+        <v>515</v>
       </c>
       <c r="G2" s="31" t="s">
-        <v>533</v>
+        <v>516</v>
       </c>
       <c r="H2" s="31" t="s">
-        <v>534</v>
+        <v>517</v>
       </c>
       <c r="I2" s="31" t="s">
-        <v>535</v>
+        <v>518</v>
       </c>
       <c r="J2" s="30" t="s">
-        <v>536</v>
+        <v>519</v>
       </c>
       <c r="K2" s="31" t="s">
-        <v>537</v>
+        <v>520</v>
       </c>
       <c r="L2" s="31" t="s">
-        <v>538</v>
+        <v>521</v>
       </c>
       <c r="M2" s="31" t="s">
-        <v>539</v>
+        <v>522</v>
       </c>
       <c r="N2" s="30" t="s">
-        <v>540</v>
+        <v>523</v>
       </c>
       <c r="O2" s="31" t="s">
         <v>52</v>
@@ -7546,7 +7549,7 @@
     </row>
     <row r="3" spans="1:15" ht="16" x14ac:dyDescent="0.2">
       <c r="A3" s="29" t="s">
-        <v>586</v>
+        <v>567</v>
       </c>
       <c r="B3" s="29" t="s">
         <v>15</v>
@@ -7588,7 +7591,7 @@
     </row>
     <row r="4" spans="1:15" ht="80" x14ac:dyDescent="0.2">
       <c r="A4" s="29" t="s">
-        <v>587</v>
+        <v>568</v>
       </c>
       <c r="B4" s="29" t="s">
         <v>15</v>
@@ -7620,12 +7623,12 @@
         <v>55</v>
       </c>
       <c r="O4" s="31" t="s">
-        <v>541</v>
+        <v>524</v>
       </c>
     </row>
     <row r="5" spans="1:15" ht="112" x14ac:dyDescent="0.2">
       <c r="A5" s="29" t="s">
-        <v>588</v>
+        <v>569</v>
       </c>
       <c r="B5" s="29" t="s">
         <v>15</v>
@@ -7665,7 +7668,7 @@
       </c>
       <c r="N5" s="31"/>
       <c r="O5" s="31" t="s">
-        <v>542</v>
+        <v>525</v>
       </c>
     </row>
   </sheetData>
@@ -7750,7 +7753,7 @@
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
-        <v>600</v>
+        <v>581</v>
       </c>
       <c r="B3" s="2" t="s">
         <v>15</v>
@@ -7759,10 +7762,10 @@
         <v>2541</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>543</v>
+        <v>526</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>544</v>
+        <v>527</v>
       </c>
       <c r="F3" s="2">
         <v>10</v>
@@ -7779,7 +7782,7 @@
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A4" s="2" t="s">
-        <v>601</v>
+        <v>582</v>
       </c>
       <c r="B4" s="2" t="s">
         <v>15</v>
@@ -7788,10 +7791,10 @@
         <v>2441</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>545</v>
+        <v>528</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>546</v>
+        <v>529</v>
       </c>
       <c r="F4" s="2">
         <v>8</v>
@@ -7808,7 +7811,7 @@
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A5" s="2" t="s">
-        <v>602</v>
+        <v>583</v>
       </c>
       <c r="B5" s="2" t="s">
         <v>15</v>
@@ -7817,10 +7820,10 @@
         <v>2148</v>
       </c>
       <c r="D5" t="s">
-        <v>547</v>
+        <v>530</v>
       </c>
       <c r="E5" t="s">
-        <v>548</v>
+        <v>531</v>
       </c>
       <c r="F5">
         <v>9</v>
@@ -7837,7 +7840,7 @@
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A6" s="2" t="s">
-        <v>603</v>
+        <v>584</v>
       </c>
       <c r="B6" s="2" t="s">
         <v>15</v>
@@ -7846,10 +7849,10 @@
         <v>2372</v>
       </c>
       <c r="D6" t="s">
-        <v>549</v>
+        <v>532</v>
       </c>
       <c r="E6" t="s">
-        <v>550</v>
+        <v>533</v>
       </c>
       <c r="F6">
         <v>9</v>
@@ -7866,7 +7869,7 @@
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A7" s="2" t="s">
-        <v>604</v>
+        <v>585</v>
       </c>
       <c r="B7" s="2" t="s">
         <v>15</v>
@@ -7875,10 +7878,10 @@
         <v>2800</v>
       </c>
       <c r="D7" t="s">
-        <v>551</v>
+        <v>534</v>
       </c>
       <c r="E7" t="s">
-        <v>552</v>
+        <v>535</v>
       </c>
       <c r="F7">
         <v>9</v>
@@ -7895,7 +7898,7 @@
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A8" s="2" t="s">
-        <v>605</v>
+        <v>586</v>
       </c>
       <c r="B8" s="2" t="s">
         <v>15</v>
@@ -7904,10 +7907,10 @@
         <v>2476</v>
       </c>
       <c r="D8" t="s">
-        <v>553</v>
+        <v>536</v>
       </c>
       <c r="E8" t="s">
-        <v>554</v>
+        <v>537</v>
       </c>
       <c r="F8">
         <v>9</v>
@@ -7924,7 +7927,7 @@
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A9" s="2" t="s">
-        <v>606</v>
+        <v>587</v>
       </c>
       <c r="B9" s="2" t="s">
         <v>15</v>
@@ -7933,10 +7936,10 @@
         <v>2024</v>
       </c>
       <c r="D9" t="s">
-        <v>555</v>
+        <v>538</v>
       </c>
       <c r="E9" t="s">
-        <v>556</v>
+        <v>539</v>
       </c>
       <c r="F9">
         <v>9</v>
@@ -7990,7 +7993,7 @@
         <v>427</v>
       </c>
       <c r="D1" s="9" t="s">
-        <v>557</v>
+        <v>540</v>
       </c>
       <c r="E1" s="9" t="s">
         <v>169</v>
@@ -8002,13 +8005,13 @@
         <v>166</v>
       </c>
       <c r="H1" s="9" t="s">
-        <v>558</v>
+        <v>541</v>
       </c>
       <c r="I1" s="9" t="s">
-        <v>559</v>
+        <v>542</v>
       </c>
       <c r="J1" s="9" t="s">
-        <v>560</v>
+        <v>543</v>
       </c>
       <c r="K1" s="9" t="s">
         <v>39</v>
@@ -8022,28 +8025,28 @@
         <v>8</v>
       </c>
       <c r="C2" t="s">
-        <v>561</v>
+        <v>544</v>
       </c>
       <c r="D2" s="9" t="s">
-        <v>562</v>
+        <v>545</v>
       </c>
       <c r="E2" s="9" t="s">
-        <v>563</v>
+        <v>546</v>
       </c>
       <c r="F2" s="9" t="s">
-        <v>564</v>
+        <v>547</v>
       </c>
       <c r="G2" s="9" t="s">
-        <v>565</v>
+        <v>548</v>
       </c>
       <c r="H2" s="9" t="s">
-        <v>566</v>
+        <v>549</v>
       </c>
       <c r="I2" s="9" t="s">
-        <v>567</v>
+        <v>550</v>
       </c>
       <c r="J2" s="9" t="s">
-        <v>568</v>
+        <v>551</v>
       </c>
       <c r="K2" s="9" t="s">
         <v>52</v>
@@ -8051,7 +8054,7 @@
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>569</v>
+        <v>605</v>
       </c>
       <c r="B3" t="s">
         <v>15</v>
@@ -8083,7 +8086,7 @@
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>570</v>
+        <v>606</v>
       </c>
       <c r="B4" t="s">
         <v>15</v>
@@ -8113,7 +8116,7 @@
         <v>16</v>
       </c>
       <c r="K4" s="9" t="s">
-        <v>571</v>
+        <v>552</v>
       </c>
     </row>
   </sheetData>
@@ -8362,7 +8365,7 @@
         <v>2</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>572</v>
+        <v>553</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.2">
@@ -8370,7 +8373,7 @@
         <v>137</v>
       </c>
       <c r="B2" t="s">
-        <v>573</v>
+        <v>554</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.2">
@@ -8378,7 +8381,7 @@
         <v>2431</v>
       </c>
       <c r="B3" t="s">
-        <v>574</v>
+        <v>555</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.2">
@@ -8386,7 +8389,7 @@
         <v>2890</v>
       </c>
       <c r="B4" t="s">
-        <v>574</v>
+        <v>555</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.2">
@@ -8394,7 +8397,7 @@
         <v>2898</v>
       </c>
       <c r="B5" t="s">
-        <v>574</v>
+        <v>555</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.2">
@@ -8402,7 +8405,7 @@
         <v>2339</v>
       </c>
       <c r="B6" t="s">
-        <v>575</v>
+        <v>556</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.2">
@@ -8410,7 +8413,7 @@
         <v>2342</v>
       </c>
       <c r="B7" t="s">
-        <v>575</v>
+        <v>556</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.2">
@@ -8418,7 +8421,7 @@
         <v>2379</v>
       </c>
       <c r="B8" t="s">
-        <v>575</v>
+        <v>556</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.2">
@@ -8426,7 +8429,7 @@
         <v>2000</v>
       </c>
       <c r="B9" t="s">
-        <v>576</v>
+        <v>557</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.2">
@@ -8434,7 +8437,7 @@
         <v>2128</v>
       </c>
       <c r="B10" t="s">
-        <v>576</v>
+        <v>557</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.2">
@@ -8442,7 +8445,7 @@
         <v>2839</v>
       </c>
       <c r="B11" t="s">
-        <v>576</v>
+        <v>557</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.2">
@@ -8450,7 +8453,7 @@
         <v>2354</v>
       </c>
       <c r="B12" t="s">
-        <v>577</v>
+        <v>558</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.2">
@@ -8458,7 +8461,7 @@
         <v>2359</v>
       </c>
       <c r="B13" t="s">
-        <v>577</v>
+        <v>558</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.2">
@@ -8466,7 +8469,7 @@
         <v>2475</v>
       </c>
       <c r="B14" t="s">
-        <v>577</v>
+        <v>558</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.2">
@@ -8474,7 +8477,7 @@
         <v>2350</v>
       </c>
       <c r="B15" t="s">
-        <v>578</v>
+        <v>559</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.2">
@@ -8482,7 +8485,7 @@
         <v>2368</v>
       </c>
       <c r="B16" t="s">
-        <v>578</v>
+        <v>559</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.2">
@@ -8490,7 +8493,7 @@
         <v>2580</v>
       </c>
       <c r="B17" t="s">
-        <v>578</v>
+        <v>559</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.2">
@@ -8498,7 +8501,7 @@
         <v>2365</v>
       </c>
       <c r="B18" t="s">
-        <v>579</v>
+        <v>560</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.2">
@@ -8506,7 +8509,7 @@
         <v>2624</v>
       </c>
       <c r="B19" t="s">
-        <v>579</v>
+        <v>560</v>
       </c>
     </row>
   </sheetData>
@@ -8528,7 +8531,7 @@
         <v>137</v>
       </c>
       <c r="B1" t="s">
-        <v>580</v>
+        <v>561</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.2">
@@ -8536,7 +8539,7 @@
         <v>2000</v>
       </c>
       <c r="B2" t="s">
-        <v>581</v>
+        <v>562</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.2">
@@ -8544,7 +8547,7 @@
         <v>2431</v>
       </c>
       <c r="B3" t="s">
-        <v>581</v>
+        <v>562</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.2">
@@ -8552,7 +8555,7 @@
         <v>2890</v>
       </c>
       <c r="B4" t="s">
-        <v>581</v>
+        <v>562</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.2">
@@ -8560,7 +8563,7 @@
         <v>2898</v>
       </c>
       <c r="B5" t="s">
-        <v>581</v>
+        <v>562</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.2">
@@ -8568,7 +8571,7 @@
         <v>2339</v>
       </c>
       <c r="B6" t="s">
-        <v>581</v>
+        <v>562</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.2">
@@ -8576,7 +8579,7 @@
         <v>2342</v>
       </c>
       <c r="B7" t="s">
-        <v>581</v>
+        <v>562</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.2">
@@ -8584,7 +8587,7 @@
         <v>2379</v>
       </c>
       <c r="B8" t="s">
-        <v>581</v>
+        <v>562</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.2">
@@ -8592,7 +8595,7 @@
         <v>2000</v>
       </c>
       <c r="B9" t="s">
-        <v>581</v>
+        <v>562</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.2">
@@ -8600,7 +8603,7 @@
         <v>2128</v>
       </c>
       <c r="B10" t="s">
-        <v>581</v>
+        <v>562</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.2">
@@ -8608,7 +8611,7 @@
         <v>2839</v>
       </c>
       <c r="B11" t="s">
-        <v>581</v>
+        <v>562</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.2">
@@ -8616,7 +8619,7 @@
         <v>2354</v>
       </c>
       <c r="B12" t="s">
-        <v>581</v>
+        <v>562</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.2">
@@ -8624,7 +8627,7 @@
         <v>2359</v>
       </c>
       <c r="B13" t="s">
-        <v>581</v>
+        <v>562</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.2">
@@ -8632,7 +8635,7 @@
         <v>2475</v>
       </c>
       <c r="B14" t="s">
-        <v>581</v>
+        <v>562</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.2">
@@ -8640,7 +8643,7 @@
         <v>2350</v>
       </c>
       <c r="B15" t="s">
-        <v>581</v>
+        <v>562</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.2">
@@ -8648,7 +8651,7 @@
         <v>2368</v>
       </c>
       <c r="B16" t="s">
-        <v>581</v>
+        <v>562</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.2">
@@ -8656,7 +8659,7 @@
         <v>2580</v>
       </c>
       <c r="B17" t="s">
-        <v>581</v>
+        <v>562</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.2">
@@ -8664,7 +8667,7 @@
         <v>2365</v>
       </c>
       <c r="B18" t="s">
-        <v>581</v>
+        <v>562</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.2">
@@ -8672,7 +8675,7 @@
         <v>2624</v>
       </c>
       <c r="B19" t="s">
-        <v>581</v>
+        <v>562</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.2">
@@ -8680,7 +8683,7 @@
         <v>3000</v>
       </c>
       <c r="B20" t="s">
-        <v>582</v>
+        <v>563</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.2">
@@ -8688,7 +8691,7 @@
         <v>3421</v>
       </c>
       <c r="B21" t="s">
-        <v>582</v>
+        <v>563</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.2">
@@ -8696,7 +8699,7 @@
         <v>3519</v>
       </c>
       <c r="B22" t="s">
-        <v>582</v>
+        <v>563</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.2">
@@ -8704,7 +8707,7 @@
         <v>4173</v>
       </c>
       <c r="B23" t="s">
-        <v>582</v>
+        <v>563</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.2">
@@ -8712,7 +8715,7 @@
         <v>4596</v>
       </c>
       <c r="B24" t="s">
-        <v>582</v>
+        <v>563</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
[DG22-2638] refactor the way to construct and run each test case scenario in all certificate activities
</commit_message>
<xml_diff>
--- a/packages/test/cypress/fixtures/data.xlsx
+++ b/packages/test/cypress/fixtures/data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/felix/kororo/repository/safeguard-github/rules-interface/packages/test/cypress/fixtures/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6B601236-50CA-B344-9AD8-0A27181D4257}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3B973134-6F47-3748-B153-74D7125EB7E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="38400" windowHeight="21100" tabRatio="816" firstSheet="10" activeTab="28" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="38400" windowHeight="21100" tabRatio="816" firstSheet="10" activeTab="27" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="BESS2_C" sheetId="11" r:id="rId1"/>
@@ -10338,12 +10338,18 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="ca5ba3f9-dfeb-4931-84ba-86796a0d6823">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <_ip_UnifiedCompliancePolicyUIAction xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
+    <DAte xmlns="ca5ba3f9-dfeb-4931-84ba-86796a0d6823" xsi:nil="true"/>
+    <_ip_UnifiedCompliancePolicyProperties xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
+    <date0 xmlns="ca5ba3f9-dfeb-4931-84ba-86796a0d6823" xsi:nil="true"/>
+    <TaxCatchAll xmlns="9ea08096-1d6a-4225-8886-dcb3dd04c4bd" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -10636,24 +10642,22 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="ca5ba3f9-dfeb-4931-84ba-86796a0d6823">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <_ip_UnifiedCompliancePolicyUIAction xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
-    <DAte xmlns="ca5ba3f9-dfeb-4931-84ba-86796a0d6823" xsi:nil="true"/>
-    <_ip_UnifiedCompliancePolicyProperties xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
-    <date0 xmlns="ca5ba3f9-dfeb-4931-84ba-86796a0d6823" xsi:nil="true"/>
-    <TaxCatchAll xmlns="9ea08096-1d6a-4225-8886-dcb3dd04c4bd" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6A69F337-BFDC-4B9A-9645-ACD2998E51C5}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3F5E14B5-D6EF-401C-82ED-6CA5F26974B2}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="ca5ba3f9-dfeb-4931-84ba-86796a0d6823"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
+    <ds:schemaRef ds:uri="9ea08096-1d6a-4225-8886-dcb3dd04c4bd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -10680,13 +10684,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3F5E14B5-D6EF-401C-82ED-6CA5F26974B2}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6A69F337-BFDC-4B9A-9645-ACD2998E51C5}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="ca5ba3f9-dfeb-4931-84ba-86796a0d6823"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
-    <ds:schemaRef ds:uri="9ea08096-1d6a-4225-8886-dcb3dd04c4bd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
[DG22-2696] adjust data auto testing
</commit_message>
<xml_diff>
--- a/packages/test/cypress/fixtures/data.xlsx
+++ b/packages/test/cypress/fixtures/data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/felix/kororo/repository/safeguard-github/rules-interface/packages/test/cypress/fixtures/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3C12D2BE-FDEE-EC4B-B60B-DB235242085A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D0BA4600-84E4-134A-AAC7-A1B7FCB1A12A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="38400" windowHeight="21100" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="38400" windowHeight="21100" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="D17_C" sheetId="10" r:id="rId1"/>
@@ -1515,9 +1515,6 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BE7981E0-7582-47E2-8222-6AD74E67DB3E}">
-  <sheetPr>
-    <tabColor rgb="FFFFFFFF"/>
-  </sheetPr>
   <dimension ref="A1:P6"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
@@ -4935,10 +4932,10 @@
         <v>114</v>
       </c>
       <c r="H5">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="I5">
-        <v>41.29</v>
+        <v>37.79</v>
       </c>
     </row>
   </sheetData>
@@ -5853,12 +5850,18 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="ca5ba3f9-dfeb-4931-84ba-86796a0d6823">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <_ip_UnifiedCompliancePolicyUIAction xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
+    <DAte xmlns="ca5ba3f9-dfeb-4931-84ba-86796a0d6823" xsi:nil="true"/>
+    <_ip_UnifiedCompliancePolicyProperties xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
+    <date0 xmlns="ca5ba3f9-dfeb-4931-84ba-86796a0d6823" xsi:nil="true"/>
+    <TaxCatchAll xmlns="9ea08096-1d6a-4225-8886-dcb3dd04c4bd" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -6151,24 +6154,22 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="ca5ba3f9-dfeb-4931-84ba-86796a0d6823">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <_ip_UnifiedCompliancePolicyUIAction xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
-    <DAte xmlns="ca5ba3f9-dfeb-4931-84ba-86796a0d6823" xsi:nil="true"/>
-    <_ip_UnifiedCompliancePolicyProperties xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
-    <date0 xmlns="ca5ba3f9-dfeb-4931-84ba-86796a0d6823" xsi:nil="true"/>
-    <TaxCatchAll xmlns="9ea08096-1d6a-4225-8886-dcb3dd04c4bd" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6A69F337-BFDC-4B9A-9645-ACD2998E51C5}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3F5E14B5-D6EF-401C-82ED-6CA5F26974B2}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="ca5ba3f9-dfeb-4931-84ba-86796a0d6823"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
+    <ds:schemaRef ds:uri="9ea08096-1d6a-4225-8886-dcb3dd04c4bd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -6195,13 +6196,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3F5E14B5-D6EF-401C-82ED-6CA5F26974B2}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6A69F337-BFDC-4B9A-9645-ACD2998E51C5}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="ca5ba3f9-dfeb-4931-84ba-86796a0d6823"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
-    <ds:schemaRef ds:uri="9ea08096-1d6a-4225-8886-dcb3dd04c4bd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
[DG22-2638] adjust test data fixture
</commit_message>
<xml_diff>
--- a/packages/test/cypress/fixtures/data.xlsx
+++ b/packages/test/cypress/fixtures/data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/felix/kororo/repository/safeguard-github/rules-interface/packages/test/cypress/fixtures/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3033BF25-D51C-364A-95FA-3AD0F83F42BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{07416A6D-DC8D-E74C-AEBE-C8C56A1F3598}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="38400" windowHeight="21100" tabRatio="816" firstSheet="5" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="38400" windowHeight="21100" tabRatio="816" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="BESS2_C" sheetId="11" r:id="rId1"/>
@@ -2840,10 +2840,10 @@
         <v>145</v>
       </c>
       <c r="H5" s="2">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="I5" s="2">
-        <v>37.79</v>
+        <v>41.29</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.2">
@@ -2927,10 +2927,10 @@
         <v>160</v>
       </c>
       <c r="H8">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="I8">
-        <v>18.48</v>
+        <v>21.99</v>
       </c>
     </row>
   </sheetData>
@@ -10256,12 +10256,18 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="ca5ba3f9-dfeb-4931-84ba-86796a0d6823">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <_ip_UnifiedCompliancePolicyUIAction xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
+    <DAte xmlns="ca5ba3f9-dfeb-4931-84ba-86796a0d6823" xsi:nil="true"/>
+    <_ip_UnifiedCompliancePolicyProperties xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
+    <date0 xmlns="ca5ba3f9-dfeb-4931-84ba-86796a0d6823" xsi:nil="true"/>
+    <TaxCatchAll xmlns="9ea08096-1d6a-4225-8886-dcb3dd04c4bd" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -10554,24 +10560,22 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="ca5ba3f9-dfeb-4931-84ba-86796a0d6823">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <_ip_UnifiedCompliancePolicyUIAction xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
-    <DAte xmlns="ca5ba3f9-dfeb-4931-84ba-86796a0d6823" xsi:nil="true"/>
-    <_ip_UnifiedCompliancePolicyProperties xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
-    <date0 xmlns="ca5ba3f9-dfeb-4931-84ba-86796a0d6823" xsi:nil="true"/>
-    <TaxCatchAll xmlns="9ea08096-1d6a-4225-8886-dcb3dd04c4bd" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6A69F337-BFDC-4B9A-9645-ACD2998E51C5}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3F5E14B5-D6EF-401C-82ED-6CA5F26974B2}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="ca5ba3f9-dfeb-4931-84ba-86796a0d6823"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
+    <ds:schemaRef ds:uri="9ea08096-1d6a-4225-8886-dcb3dd04c4bd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -10598,13 +10602,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3F5E14B5-D6EF-401C-82ED-6CA5F26974B2}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6A69F337-BFDC-4B9A-9645-ACD2998E51C5}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="ca5ba3f9-dfeb-4931-84ba-86796a0d6823"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
-    <ds:schemaRef ds:uri="9ea08096-1d6a-4225-8886-dcb3dd04c4bd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>